<commit_message>
Award test cases till Activation
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{0E4FCCB2-C068-41D3-9802-C231C898049D}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{594EBA1D-7B87-42CB-897A-7E225901AA87}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7635" activeTab="4" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
@@ -17,7 +17,8 @@
     <sheet name="Payment Request Schedule" sheetId="2" r:id="rId2"/>
     <sheet name="Progress Report Schedule" sheetId="3" r:id="rId3"/>
     <sheet name="Risk Assessment" sheetId="4" r:id="rId4"/>
-    <sheet name="Site Visit" sheetId="5" r:id="rId5"/>
+    <sheet name="Reviewer" sheetId="6" r:id="rId5"/>
+    <sheet name="Site Visit" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="73">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -221,6 +222,33 @@
   </si>
   <si>
     <t>Program &amp; Fiscal</t>
+  </si>
+  <si>
+    <t>Dropdown</t>
+  </si>
+  <si>
+    <t>ReviewerRole__c</t>
+  </si>
+  <si>
+    <t>Fiscal Reviewer</t>
+  </si>
+  <si>
+    <t>Name__c</t>
+  </si>
+  <si>
+    <t>Automation FO</t>
+  </si>
+  <si>
+    <t>Responsibility__c</t>
+  </si>
+  <si>
+    <t>Review Financial details</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>DueDate__c</t>
   </si>
 </sst>
 </file>
@@ -1101,6 +1129,92 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Updated the text input method, alert Ok method and filled the column name for inline edit
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{594EBA1D-7B87-42CB-897A-7E225901AA87}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{A768CA4E-48CA-4093-ACEC-F33F8F1949BB}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7635" activeTab="4" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21576" windowHeight="7632" activeTab="6" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Edition" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Risk Assessment" sheetId="4" r:id="rId4"/>
     <sheet name="Reviewer" sheetId="6" r:id="rId5"/>
     <sheet name="Site Visit" sheetId="5" r:id="rId6"/>
+    <sheet name="Desk Review" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="73">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -607,15 +608,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" customWidth="1"/>
     <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -629,7 +630,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -651,14 +652,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.5703125" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -672,7 +673,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -686,7 +687,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -700,7 +701,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -714,7 +715,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -737,14 +738,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.42578125" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" customWidth="1"/>
-    <col min="4" max="4" width="34.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" customWidth="1"/>
+    <col min="3" max="3" width="19.44140625" customWidth="1"/>
+    <col min="4" max="4" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -758,7 +759,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -772,7 +773,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -786,7 +787,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -800,7 +801,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -822,14 +823,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -843,7 +844,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -857,7 +858,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -871,7 +872,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -885,7 +886,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -899,7 +900,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -913,7 +914,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -927,7 +928,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -941,7 +942,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -955,7 +956,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -969,7 +970,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -983,7 +984,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -997,7 +998,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1011,7 +1012,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1025,7 +1026,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -1039,7 +1040,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -1053,7 +1054,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -1067,7 +1068,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -1081,7 +1082,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -1095,7 +1096,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -1109,7 +1110,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -1131,15 +1132,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1153,7 +1154,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1167,7 +1168,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1181,7 +1182,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1195,7 +1196,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1217,14 +1218,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.42578125" customWidth="1"/>
+    <col min="3" max="3" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1238,7 +1239,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1252,7 +1253,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1266,7 +1267,79 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
First Four test cases for Site Visit
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{A768CA4E-48CA-4093-ACEC-F33F8F1949BB}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:100000_{C7990DEA-E438-4463-8C49-3BC2A9C0C90B}" xr6:coauthVersionLast="31" xr6:coauthVersionMax="31" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21576" windowHeight="7632" activeTab="6" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="74">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -250,6 +250,9 @@
   </si>
   <si>
     <t>DueDate__c</t>
+  </si>
+  <si>
+    <t>Automation Desk Review</t>
   </si>
 </sst>
 </file>
@@ -1322,7 +1325,7 @@
         <v>57</v>
       </c>
       <c r="D2" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Funding source test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A331EE-6AFF-4805-AC75-3A3E3DDD795A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AF9F91C-2EB7-4E8E-B527-A631696740B5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21576" windowHeight="7632" firstSheet="4" activeTab="6" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21576" windowHeight="7632" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Grant_Creation" sheetId="10" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="107">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -71,9 +71,6 @@
     <t>Text</t>
   </si>
   <si>
-    <t>Automation Payment Request</t>
-  </si>
-  <si>
     <t>Frequency__c</t>
   </si>
   <si>
@@ -98,9 +95,6 @@
     <t>TextArea</t>
   </si>
   <si>
-    <t>Automation Progress Report</t>
-  </si>
-  <si>
     <t>experienceQuestion1__c</t>
   </si>
   <si>
@@ -263,97 +257,106 @@
     <t>ProjectTitle__c</t>
   </si>
   <si>
+    <t>GrantAbbreviation__c</t>
+  </si>
+  <si>
+    <t>GREG</t>
+  </si>
+  <si>
+    <t>ProjectPeriodStartDate__c</t>
+  </si>
+  <si>
+    <t>ProjectPeriodEndDate__c</t>
+  </si>
+  <si>
+    <t>BudgetCategoryPackage__c</t>
+  </si>
+  <si>
+    <t>Construction</t>
+  </si>
+  <si>
+    <t>InternalOrganization__c</t>
+  </si>
+  <si>
+    <t>SAN DIEGO ELECTRICAL TRAINING TRUST</t>
+  </si>
+  <si>
+    <t>Program__c</t>
+  </si>
+  <si>
+    <t>PG--0370</t>
+  </si>
+  <si>
+    <t>ExternalOrganization__c</t>
+  </si>
+  <si>
+    <t>Test Automation Organization</t>
+  </si>
+  <si>
+    <t>ProjectDirectorContact__c</t>
+  </si>
+  <si>
+    <t>BudgetPeriodEndDate__c</t>
+  </si>
+  <si>
+    <t>Budget</t>
+  </si>
+  <si>
+    <t>GrantType__c</t>
+  </si>
+  <si>
+    <t>Project Grant</t>
+  </si>
+  <si>
+    <t>IsMatchRequired__c</t>
+  </si>
+  <si>
+    <t>GranteeMatch__c</t>
+  </si>
+  <si>
+    <t>LaverageAllowed__c</t>
+  </si>
+  <si>
+    <t>IsProgramIncomeAnticipated__c</t>
+  </si>
+  <si>
+    <t>IsAdvancePermitted__c</t>
+  </si>
+  <si>
+    <t>IsBuildUpFunctionality__c</t>
+  </si>
+  <si>
+    <t>IsGoalsRequired__c</t>
+  </si>
+  <si>
+    <t>KPIsRequired__c</t>
+  </si>
+  <si>
+    <t>AreExpensesBuildIUpLevel__c</t>
+  </si>
+  <si>
+    <t>RiskAssessmentRequired__c</t>
+  </si>
+  <si>
+    <t>WBSRequired__c</t>
+  </si>
+  <si>
+    <t>GrantDescription__c</t>
+  </si>
+  <si>
+    <t>Assessment</t>
+  </si>
+  <si>
+    <t>Automation Progress Report Regression</t>
+  </si>
+  <si>
+    <t>Automation Payment Request Regression</t>
+  </si>
+  <si>
+    <t>Signature__c</t>
+  </si>
+  <si>
     <t>Automation Grant Regression</t>
-  </si>
-  <si>
-    <t>GrantAbbreviation__c</t>
-  </si>
-  <si>
-    <t>GREG</t>
-  </si>
-  <si>
-    <t>ProjectPeriodStartDate__c</t>
-  </si>
-  <si>
-    <t>ProjectPeriodEndDate__c</t>
-  </si>
-  <si>
-    <t>BudgetCategoryPackage__c</t>
-  </si>
-  <si>
-    <t>Construction</t>
-  </si>
-  <si>
-    <t>InternalOrganization__c</t>
-  </si>
-  <si>
-    <t>SAN DIEGO ELECTRICAL TRAINING TRUST</t>
-  </si>
-  <si>
-    <t>Program__c</t>
-  </si>
-  <si>
-    <t>PG--0370</t>
-  </si>
-  <si>
-    <t>ExternalOrganization__c</t>
-  </si>
-  <si>
-    <t>Test Automation Organization</t>
-  </si>
-  <si>
-    <t>ProjectDirectorContact__c</t>
-  </si>
-  <si>
-    <t>BudgetPeriodEndDate__c</t>
-  </si>
-  <si>
-    <t>Budget</t>
-  </si>
-  <si>
-    <t>GrantType__c</t>
-  </si>
-  <si>
-    <t>Project Grant</t>
-  </si>
-  <si>
-    <t>IsMatchRequired__c</t>
-  </si>
-  <si>
-    <t>GranteeMatch__c</t>
-  </si>
-  <si>
-    <t>LaverageAllowed__c</t>
-  </si>
-  <si>
-    <t>IsProgramIncomeAnticipated__c</t>
-  </si>
-  <si>
-    <t>IsAdvancePermitted__c</t>
-  </si>
-  <si>
-    <t>IsBuildUpFunctionality__c</t>
-  </si>
-  <si>
-    <t>IsGoalsRequired__c</t>
-  </si>
-  <si>
-    <t>KPIsRequired__c</t>
-  </si>
-  <si>
-    <t>AreExpensesBuildIUpLevel__c</t>
-  </si>
-  <si>
-    <t>RiskAssessmentRequired__c</t>
-  </si>
-  <si>
-    <t>WBSRequired__c</t>
-  </si>
-  <si>
-    <t>GrantDescription__c</t>
-  </si>
-  <si>
-    <t>Assessment</t>
   </si>
 </sst>
 </file>
@@ -734,10 +737,10 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C2" t="s">
-        <v>75</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -745,10 +748,10 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -756,7 +759,7 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -767,7 +770,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C5">
         <v>500</v>
@@ -778,10 +781,10 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -789,10 +792,10 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -800,10 +803,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -811,10 +814,10 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -847,10 +850,10 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -858,10 +861,10 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" t="s">
         <v>59</v>
-      </c>
-      <c r="C3" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -869,10 +872,10 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -906,10 +909,10 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -917,10 +920,10 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" t="s">
         <v>59</v>
-      </c>
-      <c r="C3" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -928,10 +931,10 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -987,10 +990,10 @@
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -1001,136 +1004,136 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E21" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1164,10 +1167,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1175,10 +1178,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1186,7 +1189,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C4">
         <v>10</v>
@@ -1197,10 +1200,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -1208,10 +1211,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1219,10 +1222,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1230,10 +1233,10 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -1241,10 +1244,10 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -1252,10 +1255,10 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -1263,10 +1266,10 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -1274,10 +1277,10 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1285,10 +1288,10 @@
         <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1296,10 +1299,10 @@
         <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -1307,10 +1310,10 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -1381,10 +1384,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1395,15 +1398,15 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C4">
         <v>365</v>
@@ -1420,7 +1423,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -1442,7 +1445,7 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1450,10 +1453,10 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1461,10 +1464,10 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
         <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1472,10 +1475,10 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
         <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1512,7 +1515,7 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1520,10 +1523,10 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1531,10 +1534,10 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
         <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1542,10 +1545,10 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
         <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1555,7 +1558,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.21875" bestFit="1" customWidth="1"/>
@@ -1576,222 +1579,211 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B20" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>105</v>
-      </c>
-      <c r="B21" t="s">
-        <v>55</v>
-      </c>
-      <c r="C21" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1801,7 +1793,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
@@ -1825,10 +1817,21 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1862,10 +1865,10 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1873,10 +1876,10 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1884,10 +1887,10 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1895,7 +1898,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C5">
         <v>3</v>

</xml_diff>

<commit_message>
amendment request test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AF9F91C-2EB7-4E8E-B527-A631696740B5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154E914D-DC92-417F-8F74-DAF725542A1A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21576" windowHeight="7632" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
@@ -260,9 +260,6 @@
     <t>GrantAbbreviation__c</t>
   </si>
   <si>
-    <t>GREG</t>
-  </si>
-  <si>
     <t>ProjectPeriodStartDate__c</t>
   </si>
   <si>
@@ -356,7 +353,10 @@
     <t>Signature__c</t>
   </si>
   <si>
-    <t>Automation Grant Regression</t>
+    <t>Automation Grant Award for Amendment</t>
+  </si>
+  <si>
+    <t>GGAA</t>
   </si>
 </sst>
 </file>
@@ -740,7 +740,7 @@
         <v>72</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -751,7 +751,7 @@
         <v>73</v>
       </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -759,7 +759,7 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -770,7 +770,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C5">
         <v>500</v>
@@ -781,10 +781,10 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" t="s">
         <v>77</v>
-      </c>
-      <c r="C6" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -792,10 +792,10 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" t="s">
         <v>79</v>
-      </c>
-      <c r="C7" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -803,10 +803,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" t="s">
         <v>81</v>
-      </c>
-      <c r="C8" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -814,10 +814,10 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" t="s">
         <v>83</v>
-      </c>
-      <c r="C9" t="s">
-        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1167,10 +1167,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" t="s">
         <v>88</v>
-      </c>
-      <c r="C2" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1178,7 +1178,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C3" t="s">
         <v>39</v>
@@ -1189,7 +1189,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C4">
         <v>10</v>
@@ -1200,7 +1200,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C5" t="s">
         <v>39</v>
@@ -1211,7 +1211,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
         <v>39</v>
@@ -1222,7 +1222,7 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
         <v>39</v>
@@ -1233,7 +1233,7 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C8" t="s">
         <v>32</v>
@@ -1244,7 +1244,7 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C9" t="s">
         <v>39</v>
@@ -1255,7 +1255,7 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C10" t="s">
         <v>39</v>
@@ -1266,7 +1266,7 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C11" t="s">
         <v>39</v>
@@ -1277,7 +1277,7 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C12" t="s">
         <v>39</v>
@@ -1288,7 +1288,7 @@
         <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C13" t="s">
         <v>32</v>
@@ -1299,7 +1299,7 @@
         <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C14" t="s">
         <v>59</v>
@@ -1310,7 +1310,7 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C15" t="s">
         <v>17</v>
@@ -1384,7 +1384,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
         <v>59</v>
@@ -1403,10 +1403,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C4">
         <v>365</v>
@@ -1445,7 +1445,7 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1515,7 +1515,7 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1579,7 +1579,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B2" t="s">
         <v>19</v>
@@ -1590,7 +1590,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B3" t="s">
         <v>21</v>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B4" t="s">
         <v>23</v>
@@ -1612,7 +1612,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B5" t="s">
         <v>25</v>
@@ -1623,7 +1623,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
@@ -1634,7 +1634,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" t="s">
         <v>29</v>
@@ -1645,7 +1645,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B8" t="s">
         <v>31</v>
@@ -1656,7 +1656,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B9" t="s">
         <v>33</v>
@@ -1667,7 +1667,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B10" t="s">
         <v>35</v>
@@ -1678,7 +1678,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B11" t="s">
         <v>36</v>
@@ -1689,7 +1689,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B12" t="s">
         <v>37</v>
@@ -1700,7 +1700,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B13" t="s">
         <v>38</v>
@@ -1711,7 +1711,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B14" t="s">
         <v>40</v>
@@ -1722,7 +1722,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B15" t="s">
         <v>41</v>
@@ -1733,7 +1733,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B16" t="s">
         <v>43</v>
@@ -1744,7 +1744,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B17" t="s">
         <v>44</v>
@@ -1755,7 +1755,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B18" t="s">
         <v>46</v>
@@ -1766,7 +1766,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B19" t="s">
         <v>48</v>
@@ -1777,7 +1777,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B20" t="s">
         <v>50</v>
@@ -1828,7 +1828,7 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s">
         <v>54</v>

</xml_diff>

<commit_message>
Updated Sit Visit Test Cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154E914D-DC92-417F-8F74-DAF725542A1A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E27800CA-EB6A-46D8-B758-65EC36CF2970}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21576" windowHeight="7632" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Grant_Creation" sheetId="10" r:id="rId1"/>

</xml_diff>

<commit_message>
Merged PR 2108: Merge MahadevProduct18March to master
Done changes in Progress Report module and in payment request
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D4A036-4116-415E-B9D1-766123C42AE9}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862C35A6-8DC2-473E-9E89-13E540330D13}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Grant_Creation" sheetId="10" r:id="rId1"/>
@@ -363,7 +363,7 @@
     <t>Automation Permanent Internal Program</t>
   </si>
   <si>
-    <t>Automation Grant Award for Post Award"</t>
+    <t>Automation Permanent Award</t>
   </si>
 </sst>
 </file>
@@ -738,13 +738,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
     <col min="3" max="3" width="36" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -755,7 +755,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -766,7 +766,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -777,7 +777,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -788,7 +788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -799,7 +799,7 @@
         <v>1095</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -810,7 +810,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -821,7 +821,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -832,7 +832,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -852,14 +852,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -870,7 +870,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -881,7 +881,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -892,7 +892,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -903,7 +903,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -923,13 +923,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -940,7 +940,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -951,7 +951,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -962,7 +962,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -981,14 +981,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -999,7 +999,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1010,7 +1010,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1040,18 +1040,18 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1117,7 +1117,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1151,82 +1151,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -1239,14 +1239,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1279,7 +1279,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1301,7 +1301,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1323,7 +1323,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1334,7 +1334,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1345,7 +1345,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1356,7 +1356,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1367,7 +1367,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1398,13 +1398,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1437,7 +1437,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -1486,14 +1486,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1504,7 +1504,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1515,7 +1515,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -1535,14 +1535,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1553,7 +1553,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -1583,13 +1583,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1611,7 +1611,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1644,7 +1644,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1655,7 +1655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1675,13 +1675,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1703,7 +1703,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1714,7 +1714,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1736,7 +1736,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1747,7 +1747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1767,14 +1767,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1785,7 +1785,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1796,7 +1796,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1807,7 +1807,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1862,7 +1862,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1884,7 +1884,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1895,7 +1895,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1917,7 +1917,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1939,7 +1939,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -2002,14 +2002,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2020,7 +2020,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2254: Merge MahadevProductB to master
Fixed award scenarios
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{341A580A-3038-4D5F-91CA-E9A1832FEE0F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F924BC8F-6D39-48B4-A019-D49B4DEC2B8A}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Grant_Creation" sheetId="10" r:id="rId1"/>
@@ -363,7 +363,7 @@
     <t>Automation Permanent Internal Program</t>
   </si>
   <si>
-    <t>Automation Permanent Award</t>
+    <t>Automation Execution Award</t>
   </si>
 </sst>
 </file>
@@ -796,7 +796,7 @@
         <v>72</v>
       </c>
       <c r="C5">
-        <v>1095</v>
+        <v>3650</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1364,7 +1364,7 @@
         <v>93</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -1523,7 +1523,7 @@
         <v>80</v>
       </c>
       <c r="C3">
-        <v>1095</v>
+        <v>3650</v>
       </c>
     </row>
   </sheetData>
@@ -1572,7 +1572,7 @@
         <v>80</v>
       </c>
       <c r="C3">
-        <v>1095</v>
+        <v>3650</v>
       </c>
     </row>
   </sheetData>
@@ -1663,7 +1663,7 @@
         <v>101</v>
       </c>
       <c r="C7">
-        <v>670</v>
+        <v>3650</v>
       </c>
     </row>
   </sheetData>
@@ -1755,7 +1755,7 @@
         <v>101</v>
       </c>
       <c r="C7">
-        <v>670</v>
+        <v>3650</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merged PR 2288: Merge applicationintake-refactoring to master
updated the deletion api on directed announcement
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F924BC8F-6D39-48B4-A019-D49B4DEC2B8A}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F4636D0-1A7D-430B-B318-0465AC028E44}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Grant_Creation" sheetId="10" r:id="rId1"/>
@@ -738,13 +738,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
     <col min="3" max="3" width="36" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -755,7 +755,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -766,7 +766,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -777,7 +777,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -788,7 +788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -799,7 +799,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -810,7 +810,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -821,7 +821,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -832,7 +832,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -852,14 +852,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -870,7 +870,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -881,7 +881,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -892,7 +892,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -903,7 +903,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -923,13 +923,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -940,7 +940,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -951,7 +951,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -962,7 +962,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -981,14 +981,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -999,7 +999,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1010,7 +1010,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1040,18 +1040,18 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1117,7 +1117,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1151,82 +1151,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -1239,14 +1239,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1279,7 +1279,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1301,7 +1301,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1323,7 +1323,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1334,7 +1334,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1345,7 +1345,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1356,7 +1356,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1367,7 +1367,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1398,13 +1398,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1437,7 +1437,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -1486,14 +1486,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1504,7 +1504,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1515,7 +1515,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -1523,7 +1523,7 @@
         <v>80</v>
       </c>
       <c r="C3">
-        <v>3650</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -1535,14 +1535,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1553,7 +1553,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -1583,13 +1583,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1611,7 +1611,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1644,7 +1644,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1655,7 +1655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1675,13 +1675,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1703,7 +1703,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1714,7 +1714,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1736,7 +1736,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1747,7 +1747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1767,14 +1767,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1785,7 +1785,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1796,7 +1796,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1807,7 +1807,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1862,7 +1862,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1884,7 +1884,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1895,7 +1895,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1917,7 +1917,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1939,7 +1939,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -2002,14 +2002,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2020,7 +2020,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2429: Merge MahadevProductB to master
removed consolidated steps and replaced with individual steps
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF7E4719-65A4-4E87-8AA1-42B9CAFC2C48}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DFD8002-CD5A-46BF-9E3E-BB6A129ED28F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="10" activeTab="14" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -27,7 +27,8 @@
     <sheet name="Reviewer" sheetId="6" r:id="rId12"/>
     <sheet name="Site Visit" sheetId="5" r:id="rId13"/>
     <sheet name="Desk Review" sheetId="7" r:id="rId14"/>
-    <sheet name="Sheet1" sheetId="8" r:id="rId15"/>
+    <sheet name="KPI" sheetId="18" r:id="rId15"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId16"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="113">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -369,6 +370,15 @@
   </si>
   <si>
     <t>12/09/2019</t>
+  </si>
+  <si>
+    <t>fieldMasterKPI__c</t>
+  </si>
+  <si>
+    <t>Automation Permanent KPI for Regression2</t>
+  </si>
+  <si>
+    <t>fieldTarget__c</t>
   </si>
 </sst>
 </file>
@@ -1289,6 +1299,54 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Merged PR 2487: Merge jit_prod to master
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA688ED7-4917-4FFC-9DF9-54BB534285B5}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B78901-D655-47C7-BEDA-EA2821021FBC}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="1131" yWindow="1131" windowWidth="16458" windowHeight="8555" firstSheet="4" activeTab="5" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -759,13 +759,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -776,7 +776,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -787,7 +787,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -798,7 +798,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -809,7 +809,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -820,7 +820,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -840,14 +840,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -858,7 +858,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -869,7 +869,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -880,7 +880,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -891,7 +891,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -902,7 +902,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -913,7 +913,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -924,7 +924,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -935,7 +935,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -946,7 +946,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -957,7 +957,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -968,7 +968,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -979,7 +979,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -990,7 +990,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1001,7 +1001,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1012,7 +1012,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1023,7 +1023,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1034,7 +1034,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1056,7 +1056,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1075,14 +1075,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.07421875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.4609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1113,14 +1113,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1131,7 +1131,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1142,7 +1142,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1153,7 +1153,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1164,7 +1164,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1184,13 +1184,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.4609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1201,7 +1201,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1212,7 +1212,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1223,7 +1223,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1242,14 +1242,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1301,13 +1301,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" customWidth="1"/>
+    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.07421875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1318,7 +1318,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1329,7 +1329,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1349,18 +1349,18 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.4609375" customWidth="1"/>
+    <col min="2" max="2" width="9.69140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="4" max="4" width="10.3046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.07421875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.4609375" customWidth="1"/>
+    <col min="7" max="7" width="13.4609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1383,7 +1383,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1460,82 +1460,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -1548,13 +1548,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1565,7 +1565,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1576,7 +1576,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1598,7 +1598,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1609,7 +1609,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1629,13 +1629,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
-    <col min="3" max="3" width="39.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.07421875" customWidth="1"/>
+    <col min="3" max="3" width="39.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1668,7 +1668,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1690,7 +1690,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1701,7 +1701,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1723,7 +1723,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1743,14 +1743,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.69140625" customWidth="1"/>
+    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1761,7 +1761,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1772,7 +1772,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1794,7 +1794,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1805,7 +1805,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1816,7 +1816,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1827,7 +1827,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1838,7 +1838,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1849,7 +1849,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1860,7 +1860,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1871,7 +1871,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1902,13 +1902,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1930,7 +1930,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1941,7 +1941,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1974,7 +1974,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -1990,14 +1990,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.69140625" customWidth="1"/>
+    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2019,7 +2019,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2027,7 +2027,7 @@
         <v>80</v>
       </c>
       <c r="C3">
-        <v>200</v>
+        <v>1200</v>
       </c>
     </row>
   </sheetData>
@@ -2039,14 +2039,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.69140625" customWidth="1"/>
+    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2087,13 +2087,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2115,7 +2115,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2126,7 +2126,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2137,7 +2137,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2148,7 +2148,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2159,7 +2159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2179,13 +2179,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2196,7 +2196,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2207,7 +2207,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2229,7 +2229,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2240,7 +2240,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2251,7 +2251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2494: Merge MahadevProductB to master
ProjectManager.java - Added new method to verify total records in flex table
PaymentRequest.feature - moved scenario @53838 to award feature file
subawardStandAlone.feature - Added 4 new scenarios

Related work items: #53837, #53911, #53838, #53910, #53840
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B78901-D655-47C7-BEDA-EA2821021FBC}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52A9CFD-8B45-4474-8957-80849ADC2674}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1131" yWindow="1131" windowWidth="16458" windowHeight="8555" firstSheet="4" activeTab="5" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="11" activeTab="16" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -29,6 +29,7 @@
     <sheet name="Desk Review" sheetId="7" r:id="rId14"/>
     <sheet name="KPI" sheetId="18" r:id="rId15"/>
     <sheet name="Sheet1" sheetId="8" r:id="rId16"/>
+    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId17"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="114">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -379,13 +380,27 @@
   </si>
   <si>
     <t>Automation Execution Award</t>
+  </si>
+  <si>
+    <r>
+      <t>09/24/2022</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -410,6 +425,26 @@
       <color rgb="FF000000"/>
       <name val="Helvetica"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF4E586A"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -431,7 +466,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -444,6 +479,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -759,13 +803,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -776,7 +820,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -787,7 +831,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -798,7 +842,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -809,7 +853,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -820,7 +864,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -840,14 +884,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -858,7 +902,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -869,7 +913,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -880,7 +924,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -891,7 +935,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -902,7 +946,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -913,7 +957,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -924,7 +968,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -935,7 +979,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -946,7 +990,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -957,7 +1001,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -968,7 +1012,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -979,7 +1023,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -990,7 +1034,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1001,7 +1045,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1012,7 +1056,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1023,7 +1067,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1034,7 +1078,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1045,7 +1089,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1056,7 +1100,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1075,14 +1119,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.4609375" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1093,7 +1137,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1113,14 +1157,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1131,7 +1175,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1142,7 +1186,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1153,7 +1197,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1164,7 +1208,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1184,13 +1228,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.4609375" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1201,7 +1245,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1212,7 +1256,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1223,7 +1267,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1242,14 +1286,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1260,7 +1304,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1271,7 +1315,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1282,7 +1326,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1301,13 +1345,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.07421875" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1318,7 +1362,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1329,7 +1373,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1349,18 +1393,18 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.4609375" customWidth="1"/>
-    <col min="2" max="2" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.3046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.07421875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.4609375" customWidth="1"/>
-    <col min="7" max="7" width="13.4609375" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1383,7 +1427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1406,7 +1450,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1426,7 +1470,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1446,7 +1490,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1460,84 +1504,241 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1548,13 +1749,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1565,7 +1766,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1576,7 +1777,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1587,7 +1788,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1598,7 +1799,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1609,7 +1810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1629,13 +1830,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.07421875" customWidth="1"/>
-    <col min="3" max="3" width="39.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="3" width="39.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1646,7 +1847,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1657,7 +1858,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1668,7 +1869,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1679,7 +1880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1690,7 +1891,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1701,7 +1902,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1712,7 +1913,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1723,7 +1924,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1743,14 +1944,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.69140625" customWidth="1"/>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1761,7 +1962,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1772,7 +1973,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1783,7 +1984,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1794,7 +1995,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1805,7 +2006,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1816,7 +2017,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1827,7 +2028,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1838,7 +2039,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1849,7 +2050,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1860,7 +2061,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1871,7 +2072,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1882,7 +2083,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1902,13 +2103,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.53515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -1919,7 +2120,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1930,7 +2131,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1941,7 +2142,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -1952,7 +2153,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1963,7 +2164,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1974,7 +2175,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -1989,15 +2190,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2008,7 +2209,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2019,16 +2220,22 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
       <c r="B3" t="s">
         <v>80</v>
       </c>
-      <c r="C3">
-        <v>1200</v>
-      </c>
+      <c r="C3" s="6" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" s="7"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2039,14 +2246,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2057,7 +2264,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2068,7 +2275,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2087,13 +2294,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2104,7 +2311,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2115,7 +2322,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2126,7 +2333,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2137,7 +2344,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2148,7 +2355,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2159,7 +2366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2179,13 +2386,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2196,7 +2403,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2207,7 +2414,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2218,7 +2425,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2229,7 +2436,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2240,7 +2447,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2251,7 +2458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2495: Merge jit_prod to master
Refactored award FDM
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52A9CFD-8B45-4474-8957-80849ADC2674}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C36D46B-1788-4D42-8FE2-7927E229B0E8}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="11" activeTab="16" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="1131" yWindow="1131" windowWidth="16458" windowHeight="8555" activeTab="1" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -29,7 +29,6 @@
     <sheet name="Desk Review" sheetId="7" r:id="rId14"/>
     <sheet name="KPI" sheetId="18" r:id="rId15"/>
     <sheet name="Sheet1" sheetId="8" r:id="rId16"/>
-    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId17"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="114">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -367,9 +366,6 @@
     <t>Automation Permanent Internal Program</t>
   </si>
   <si>
-    <t>12/09/2019</t>
-  </si>
-  <si>
     <t>fieldMasterKPI__c</t>
   </si>
   <si>
@@ -382,25 +378,17 @@
     <t>Automation Execution Award</t>
   </si>
   <si>
-    <r>
-      <t>09/24/2022</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Segoe UI"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
+    <t>09/24/2022</t>
+  </si>
+  <si>
+    <t>09/23/2022</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -425,26 +413,6 @@
       <color rgb="FF000000"/>
       <name val="Helvetica"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FF4E586A"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -466,7 +434,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -479,15 +447,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -803,13 +763,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -820,7 +780,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -831,7 +791,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -842,7 +802,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -853,7 +813,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -864,7 +824,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -872,7 +832,7 @@
         <v>101</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -884,14 +844,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -902,7 +862,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -913,7 +873,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -924,7 +884,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -935,7 +895,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -946,7 +906,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -957,7 +917,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -968,7 +928,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -979,7 +939,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -990,7 +950,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1001,7 +961,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1012,7 +972,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1023,7 +983,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1034,7 +994,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1045,7 +1005,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1056,7 +1016,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1067,7 +1027,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1078,7 +1038,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1089,7 +1049,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1100,7 +1060,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1119,14 +1079,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.07421875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.4609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1137,7 +1097,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1157,14 +1117,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1175,7 +1135,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1186,7 +1146,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1197,7 +1157,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1208,7 +1168,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1228,13 +1188,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.4609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1245,7 +1205,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1256,7 +1216,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1267,7 +1227,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1286,14 +1246,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1304,7 +1264,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1315,7 +1275,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1326,7 +1286,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1345,13 +1305,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.07421875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1362,23 +1322,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>110</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>111</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1393,18 +1353,18 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.4609375" customWidth="1"/>
+    <col min="2" max="2" width="9.69140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="10.3046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.07421875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.4609375" customWidth="1"/>
+    <col min="7" max="7" width="13.4609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1427,7 +1387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1450,7 +1410,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1470,7 +1430,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1490,7 +1450,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1504,241 +1464,84 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E21" t="s">
         <v>51</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>89</v>
-      </c>
-      <c r="C7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>93</v>
-      </c>
-      <c r="C11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C13" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1749,13 +1552,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1766,7 +1569,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1777,7 +1580,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1788,7 +1591,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1799,7 +1602,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1810,7 +1613,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1818,7 +1621,7 @@
         <v>101</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1830,13 +1633,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
-    <col min="3" max="3" width="39.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.07421875" customWidth="1"/>
+    <col min="3" max="3" width="39.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1847,7 +1650,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1855,10 +1658,10 @@
         <v>69</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1869,7 +1672,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1880,7 +1683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1891,7 +1694,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1902,7 +1705,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1913,7 +1716,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1924,7 +1727,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1944,14 +1747,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.69140625" customWidth="1"/>
+    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1962,7 +1765,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1973,7 +1776,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1984,7 +1787,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1995,7 +1798,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2006,7 +1809,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2017,7 +1820,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2028,7 +1831,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2039,7 +1842,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2050,7 +1853,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2061,7 +1864,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2072,7 +1875,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2083,7 +1886,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -2103,13 +1906,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -2120,7 +1923,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2131,7 +1934,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2142,7 +1945,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -2153,7 +1956,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -2164,7 +1967,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -2175,7 +1978,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -2190,15 +1993,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.69140625" customWidth="1"/>
+    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2209,7 +2012,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2220,7 +2023,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2228,14 +2031,8 @@
         <v>80</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C5" s="7"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C6" s="8"/>
+        <v>112</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2246,14 +2043,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.69140625" customWidth="1"/>
+    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2264,7 +2061,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2275,7 +2072,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2294,13 +2091,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2311,7 +2108,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2322,7 +2119,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2333,7 +2130,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2344,7 +2141,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2355,7 +2152,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2366,7 +2163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2386,13 +2183,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2403,7 +2200,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2414,7 +2211,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2425,7 +2222,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2436,7 +2233,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2447,7 +2244,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2458,7 +2255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2514: Merge MahadevProductB to master
subawardStandAlone.feature - moved sceario " @53910"  to new feature file coz it doesn't require any background
paymentRequest_Without_Background.feature - created new feature file where scenarios doesn't require any background
paymentRequest.feature - modified one step as required and added two new scenarios

Related work items: #53969, #53966, #53971
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C36D46B-1788-4D42-8FE2-7927E229B0E8}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52A9CFD-8B45-4474-8957-80849ADC2674}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1131" yWindow="1131" windowWidth="16458" windowHeight="8555" activeTab="1" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="11" activeTab="16" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -29,6 +29,7 @@
     <sheet name="Desk Review" sheetId="7" r:id="rId14"/>
     <sheet name="KPI" sheetId="18" r:id="rId15"/>
     <sheet name="Sheet1" sheetId="8" r:id="rId16"/>
+    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId17"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="114">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -366,6 +367,9 @@
     <t>Automation Permanent Internal Program</t>
   </si>
   <si>
+    <t>12/09/2019</t>
+  </si>
+  <si>
     <t>fieldMasterKPI__c</t>
   </si>
   <si>
@@ -378,17 +382,25 @@
     <t>Automation Execution Award</t>
   </si>
   <si>
-    <t>09/24/2022</t>
-  </si>
-  <si>
-    <t>09/23/2022</t>
+    <r>
+      <t>09/24/2022</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -413,6 +425,26 @@
       <color rgb="FF000000"/>
       <name val="Helvetica"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF4E586A"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -434,7 +466,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -447,7 +479,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -763,13 +803,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -780,7 +820,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -791,7 +831,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -802,7 +842,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -813,7 +853,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -824,7 +864,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -832,7 +872,7 @@
         <v>101</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -844,14 +884,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -862,7 +902,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -873,7 +913,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -884,7 +924,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -895,7 +935,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -906,7 +946,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -917,7 +957,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -928,7 +968,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -939,7 +979,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -950,7 +990,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -961,7 +1001,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -972,7 +1012,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -983,7 +1023,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -994,7 +1034,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1005,7 +1045,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1016,7 +1056,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1027,7 +1067,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1038,7 +1078,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1049,7 +1089,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1060,7 +1100,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1079,14 +1119,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.4609375" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1097,7 +1137,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1117,14 +1157,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1135,7 +1175,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1146,7 +1186,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1157,7 +1197,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1168,7 +1208,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1188,13 +1228,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.4609375" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1205,7 +1245,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1216,7 +1256,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1227,7 +1267,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1246,14 +1286,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1264,7 +1304,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1275,7 +1315,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1286,7 +1326,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1305,13 +1345,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.07421875" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1322,23 +1362,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1353,18 +1393,18 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.4609375" customWidth="1"/>
-    <col min="2" max="2" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.3046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.07421875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.4609375" customWidth="1"/>
-    <col min="7" max="7" width="13.4609375" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1387,7 +1427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1410,7 +1450,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1430,7 +1470,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1450,7 +1490,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1464,84 +1504,241 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1552,13 +1749,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1569,7 +1766,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1580,7 +1777,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1591,7 +1788,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1602,7 +1799,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1613,7 +1810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1621,7 +1818,7 @@
         <v>101</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1633,13 +1830,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.07421875" customWidth="1"/>
-    <col min="3" max="3" width="39.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="3" width="39.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1650,7 +1847,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1658,10 +1855,10 @@
         <v>69</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1672,7 +1869,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1683,7 +1880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1694,7 +1891,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1705,7 +1902,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1716,7 +1913,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1727,7 +1924,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1747,14 +1944,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.69140625" customWidth="1"/>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1765,7 +1962,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1776,7 +1973,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1787,7 +1984,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1798,7 +1995,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1809,7 +2006,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1820,7 +2017,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1831,7 +2028,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1842,7 +2039,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1853,7 +2050,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1864,7 +2061,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1875,7 +2072,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1886,7 +2083,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1906,13 +2103,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.53515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -1923,7 +2120,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1934,7 +2131,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1945,7 +2142,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -1956,7 +2153,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1967,7 +2164,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1978,7 +2175,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -1993,15 +2190,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2012,7 +2209,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2023,7 +2220,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2031,8 +2228,14 @@
         <v>80</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>112</v>
-      </c>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" s="7"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2043,14 +2246,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2061,7 +2264,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2072,7 +2275,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2091,13 +2294,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2108,7 +2311,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2119,7 +2322,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2130,7 +2333,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2141,7 +2344,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2152,7 +2355,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2163,7 +2366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2183,13 +2386,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2200,7 +2403,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2211,7 +2414,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2222,7 +2425,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2233,7 +2436,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2244,7 +2447,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2255,7 +2458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2522: Merge jit_prod to master
Added test data.
Removed consolidated steps
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52A9CFD-8B45-4474-8957-80849ADC2674}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FA2FA18-FCEB-4A8E-82E7-44EE5AB9F910}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="11" activeTab="16" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" activeTab="1" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -367,9 +367,6 @@
     <t>Automation Permanent Internal Program</t>
   </si>
   <si>
-    <t>12/09/2019</t>
-  </si>
-  <si>
     <t>fieldMasterKPI__c</t>
   </si>
   <si>
@@ -394,6 +391,9 @@
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
+  </si>
+  <si>
+    <t>09/23/2022</t>
   </si>
 </sst>
 </file>
@@ -803,13 +803,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -820,7 +820,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -831,7 +831,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -842,7 +842,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -853,7 +853,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -864,7 +864,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -872,7 +872,7 @@
         <v>101</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -884,14 +884,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.15234375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -902,7 +902,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -913,7 +913,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -924,7 +924,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -935,7 +935,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -946,7 +946,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -957,7 +957,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -968,7 +968,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -979,7 +979,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -990,7 +990,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1001,7 +1001,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1012,7 +1012,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1023,7 +1023,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1034,7 +1034,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1056,7 +1056,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1067,7 +1067,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1078,7 +1078,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1089,7 +1089,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1100,7 +1100,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1119,14 +1119,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.15234375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.3828125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1157,14 +1157,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.3828125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1175,7 +1175,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1186,7 +1186,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1197,7 +1197,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1208,7 +1208,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1228,13 +1228,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.3828125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1256,7 +1256,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1267,7 +1267,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1286,14 +1286,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.3828125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.15234375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1315,7 +1315,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1326,7 +1326,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1345,13 +1345,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.15234375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1362,23 +1362,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>110</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>111</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1393,18 +1393,18 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.3828125" customWidth="1"/>
+    <col min="2" max="2" width="9.69140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="10.3046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.15234375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.3828125" customWidth="1"/>
+    <col min="7" max="7" width="13.3828125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1427,7 +1427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1450,7 +1450,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1490,7 +1490,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1504,82 +1504,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -1592,13 +1592,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.84375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1609,7 +1609,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1631,7 +1631,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1642,7 +1642,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1664,7 +1664,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1697,7 +1697,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1708,7 +1708,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1719,7 +1719,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1730,7 +1730,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1749,13 +1749,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.15234375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1777,7 +1777,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1799,7 +1799,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1810,7 +1810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>101</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1830,13 +1830,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
-    <col min="3" max="3" width="39.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.15234375" customWidth="1"/>
+    <col min="3" max="3" width="39.15234375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1855,10 +1855,10 @@
         <v>69</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1869,7 +1869,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1944,14 +1944,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.69140625" customWidth="1"/>
+    <col min="2" max="2" width="29.3828125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.15234375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1962,7 +1962,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1984,7 +1984,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2017,7 +2017,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2028,7 +2028,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2050,7 +2050,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2061,7 +2061,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2083,7 +2083,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -2103,13 +2103,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.15234375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2131,7 +2131,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -2153,7 +2153,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -2175,7 +2175,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -2191,14 +2191,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.69140625" customWidth="1"/>
+    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.15234375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2209,7 +2209,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2220,7 +2220,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2228,13 +2228,13 @@
         <v>80</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="C5" s="7"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="C6" s="8"/>
     </row>
   </sheetData>
@@ -2246,14 +2246,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.69140625" customWidth="1"/>
+    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.15234375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2264,7 +2264,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2294,13 +2294,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.15234375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2355,7 +2355,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2386,13 +2386,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2403,7 +2403,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2425,7 +2425,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2436,7 +2436,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2458,7 +2458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2643: Merge jit_prod to master
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FA2FA18-FCEB-4A8E-82E7-44EE5AB9F910}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DFA955F-06E3-4798-8F9C-75CD66A2F411}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" activeTab="1" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" activeTab="5" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -379,21 +379,10 @@
     <t>Automation Execution Award</t>
   </si>
   <si>
-    <r>
-      <t>09/24/2022</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Segoe UI"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
     <t>09/23/2022</t>
+  </si>
+  <si>
+    <t>09/24/2022</t>
   </si>
 </sst>
 </file>
@@ -872,7 +861,7 @@
         <v>101</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -1818,7 +1807,7 @@
         <v>101</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -2228,7 +2217,7 @@
         <v>80</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Merged PR 2679: Merge MahadevProductB to master
Added 6 new test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DFA955F-06E3-4798-8F9C-75CD66A2F411}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C74B291D-1003-4B3B-A385-EB85E305E632}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" activeTab="5" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="12" activeTab="17" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -30,6 +30,7 @@
     <sheet name="KPI" sheetId="18" r:id="rId15"/>
     <sheet name="Sheet1" sheetId="8" r:id="rId16"/>
     <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId17"/>
+    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId18"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="115">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -383,13 +384,16 @@
   </si>
   <si>
     <t>09/24/2022</t>
+  </si>
+  <si>
+    <t>Annually</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -434,6 +438,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Helvetica"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -455,7 +464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -477,6 +486,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -792,13 +802,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -809,7 +819,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -820,7 +830,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -831,7 +841,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -842,7 +852,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -853,7 +863,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -873,14 +883,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -891,7 +901,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -902,7 +912,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -913,7 +923,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -924,7 +934,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -935,7 +945,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -946,7 +956,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -957,7 +967,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -968,7 +978,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -979,7 +989,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -990,7 +1000,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1001,7 +1011,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1012,7 +1022,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1023,7 +1033,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1034,7 +1044,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1045,7 +1055,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1056,7 +1066,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1067,7 +1077,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1078,7 +1088,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1089,7 +1099,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1108,14 +1118,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.15234375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.3828125" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1126,7 +1136,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1146,14 +1156,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.3828125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1164,7 +1174,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1175,7 +1185,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1186,7 +1196,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1197,7 +1207,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1217,13 +1227,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.3828125" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1234,7 +1244,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1245,7 +1255,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1256,7 +1266,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1275,14 +1285,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.3828125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1293,7 +1303,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1304,7 +1314,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1315,7 +1325,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1334,13 +1344,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.15234375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1351,7 +1361,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1362,7 +1372,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1382,18 +1392,18 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.3828125" customWidth="1"/>
-    <col min="2" max="2" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.3046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.15234375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.3828125" customWidth="1"/>
-    <col min="7" max="7" width="13.3828125" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1416,7 +1426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1439,7 +1449,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1459,7 +1469,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1479,7 +1489,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1493,82 +1503,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -1581,13 +1591,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.84375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1598,7 +1608,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1609,7 +1619,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1620,7 +1630,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1631,7 +1641,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1642,7 +1652,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1653,7 +1663,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1664,7 +1674,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1675,7 +1685,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1686,7 +1696,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1697,7 +1707,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1708,7 +1718,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1719,7 +1729,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1732,19 +1742,111 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.15234375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1755,7 +1857,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1766,7 +1868,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1777,7 +1879,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1788,7 +1890,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1799,7 +1901,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1819,13 +1921,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.15234375" customWidth="1"/>
-    <col min="3" max="3" width="39.15234375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="3" width="39.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1836,7 +1938,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1847,7 +1949,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1858,7 +1960,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1869,7 +1971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1880,7 +1982,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1891,7 +1993,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1902,7 +2004,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1913,7 +2015,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1933,14 +2035,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.69140625" customWidth="1"/>
-    <col min="2" max="2" width="29.3828125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1951,7 +2053,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1962,7 +2064,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1973,7 +2075,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1984,7 +2086,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1995,7 +2097,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2006,7 +2108,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2017,7 +2119,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2028,7 +2130,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2039,7 +2141,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2050,7 +2152,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2061,7 +2163,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2072,7 +2174,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -2092,13 +2194,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.15234375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.53515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -2109,7 +2211,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2120,7 +2222,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2131,7 +2233,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -2142,7 +2244,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -2153,7 +2255,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -2164,7 +2266,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -2180,14 +2282,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2198,7 +2300,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2209,7 +2311,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2220,10 +2322,10 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C5" s="7"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C6" s="8"/>
     </row>
   </sheetData>
@@ -2235,14 +2337,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2253,7 +2355,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2264,7 +2366,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2283,13 +2385,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.15234375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2300,7 +2402,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2311,7 +2413,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2322,7 +2424,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2333,7 +2435,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2344,7 +2446,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2355,7 +2457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2375,13 +2477,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2392,7 +2494,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2403,7 +2505,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2414,7 +2516,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2425,7 +2527,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2436,7 +2538,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2447,7 +2549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2795: Merge mfixes to master
Done dynamic user selection changes and fixed scenarios in award module
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C0E9A4E-AD3A-476E-B8C5-7540C3B20F9F}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF4EB911-85E9-4A0B-B696-F3E9FA74EAFA}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" firstSheet="17" activeTab="20" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="5" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="115">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -381,12 +381,6 @@
   </si>
   <si>
     <t>Automation Execution Award</t>
-  </si>
-  <si>
-    <t>09/23/2022</t>
-  </si>
-  <si>
-    <t>09/24/2022</t>
   </si>
   <si>
     <t>Annually</t>
@@ -402,7 +396,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -426,13 +420,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Helvetica"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
@@ -473,7 +460,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -492,10 +479,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -810,14 +794,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -828,7 +812,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -839,7 +823,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -850,7 +834,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -861,7 +845,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -870,17 +854,6 @@
       </c>
       <c r="C5" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -892,14 +865,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -910,7 +883,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -921,7 +894,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -932,7 +905,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -943,7 +916,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -954,7 +927,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -965,7 +938,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -976,7 +949,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -987,7 +960,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -998,7 +971,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1009,7 +982,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1020,7 +993,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1031,7 +1004,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1042,7 +1015,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1053,7 +1026,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1064,7 +1037,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1075,7 +1048,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1086,7 +1059,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1097,7 +1070,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1108,7 +1081,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1127,14 +1100,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.15234375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.3828125" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1145,7 +1118,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1165,14 +1138,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.3828125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1183,7 +1156,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1194,7 +1167,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1205,7 +1178,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1216,7 +1189,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1236,13 +1209,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.3828125" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1253,7 +1226,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1264,7 +1237,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1275,7 +1248,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1294,14 +1267,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.3828125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1312,7 +1285,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1323,7 +1296,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1334,7 +1307,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1353,13 +1326,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.15234375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1370,7 +1343,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1381,7 +1354,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1401,18 +1374,18 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.3828125" customWidth="1"/>
-    <col min="2" max="2" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.3046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.15234375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.3828125" customWidth="1"/>
-    <col min="7" max="7" width="13.3828125" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1435,7 +1408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1458,7 +1431,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1478,7 +1451,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1498,7 +1471,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1512,82 +1485,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -1600,13 +1573,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.84375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1617,7 +1590,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1628,7 +1601,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1639,7 +1612,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1650,7 +1623,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1661,7 +1634,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1672,7 +1645,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1683,7 +1656,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1694,7 +1667,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1705,7 +1678,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1716,7 +1689,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1727,7 +1700,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1738,7 +1711,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1757,13 +1730,13 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1774,7 +1747,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1785,18 +1758,18 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="C3" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1807,7 +1780,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1818,7 +1791,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1829,7 +1802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1849,14 +1822,14 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.921875" customWidth="1"/>
-    <col min="2" max="2" width="32.69140625" customWidth="1"/>
-    <col min="3" max="3" width="49.921875" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" customWidth="1"/>
+    <col min="3" max="3" width="49.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1867,7 +1840,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1878,18 +1851,18 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="C3" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1900,7 +1873,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1911,7 +1884,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1922,7 +1895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1940,14 +1913,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.15234375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1958,7 +1931,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1969,7 +1942,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1980,7 +1953,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1991,7 +1964,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2002,16 +1975,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>112</v>
-      </c>
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="3"/>
+      <c r="C7" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2022,14 +1991,14 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.69140625" customWidth="1"/>
-    <col min="2" max="2" width="28.3828125" customWidth="1"/>
-    <col min="3" max="3" width="29.3046875" customWidth="1"/>
+    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2040,7 +2009,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2051,18 +2020,18 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="C3" s="8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2073,7 +2042,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2084,7 +2053,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2095,7 +2064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2114,14 +2083,14 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.921875" customWidth="1"/>
-    <col min="2" max="2" width="34.07421875" customWidth="1"/>
-    <col min="3" max="3" width="29.23046875" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" customWidth="1"/>
+    <col min="2" max="2" width="34.140625" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2132,7 +2101,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2143,18 +2112,18 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="C3" s="8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2165,7 +2134,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2176,7 +2145,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2187,7 +2156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2206,13 +2175,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.15234375" customWidth="1"/>
-    <col min="3" max="3" width="39.15234375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="3" width="39.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2223,7 +2192,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2234,7 +2203,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2245,7 +2214,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2256,7 +2225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2267,7 +2236,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2278,7 +2247,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2289,7 +2258,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2300,7 +2269,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2320,14 +2289,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.69140625" customWidth="1"/>
-    <col min="2" max="2" width="29.3828125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2338,7 +2307,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2349,7 +2318,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2360,7 +2329,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2371,7 +2340,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2382,7 +2351,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2393,7 +2362,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2404,7 +2373,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2415,7 +2384,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2426,7 +2395,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2437,7 +2406,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2448,7 +2417,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2459,7 +2428,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -2479,13 +2448,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.15234375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.53515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -2496,7 +2465,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2507,7 +2476,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2518,7 +2487,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -2529,7 +2498,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -2540,7 +2509,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -2551,7 +2520,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -2566,15 +2535,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2585,7 +2554,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2596,22 +2565,11 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C4" s="6"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C5" s="7"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="C6" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2622,14 +2580,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2640,7 +2598,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2651,7 +2609,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2670,13 +2628,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.15234375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2687,7 +2645,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2698,7 +2656,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2709,7 +2667,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2720,7 +2678,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2731,7 +2689,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2742,7 +2700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2762,13 +2720,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2779,7 +2737,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2790,7 +2748,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2801,7 +2759,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2812,7 +2770,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2823,7 +2781,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2834,7 +2792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2824: Merge mfixes to master
Added new test cases and  implemented one new step
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF4EB911-85E9-4A0B-B696-F3E9FA74EAFA}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C5FBED-49E9-41C6-8E8D-91119BCD7B59}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="5" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="21" activeTab="23" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -34,6 +34,9 @@
     <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId19"/>
     <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId20"/>
     <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId21"/>
+    <sheet name="Progress Report Annually" sheetId="24" r:id="rId22"/>
+    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId23"/>
+    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId24"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -45,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="117">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -390,6 +393,12 @@
   </si>
   <si>
     <t>Bi-Monthly</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Semi-Annually</t>
   </si>
 </sst>
 </file>
@@ -2172,6 +2181,275 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:C9"/>
@@ -2535,7 +2813,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" customWidth="1"/>
@@ -2543,7 +2821,7 @@
     <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2554,7 +2832,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2565,11 +2843,16 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C5" s="7"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>115</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Merged PR 2952: Merge mfixes to master
Added new test cases and updated failed test cases

Related work items: #55294, #57646, #55313, #57690, #55305, #57580, #55316
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,38 +5,39 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{970E8ECB-0E5D-457C-864E-861F55447FAC}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91F7757-9872-4062-BB93-A5495E37EAAA}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="2" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="3" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
     <sheet name="Payment Request Schedule_FDM" sheetId="15" r:id="rId2"/>
     <sheet name="Grant_Creation" sheetId="10" r:id="rId3"/>
-    <sheet name="Grant_Edition" sheetId="11" r:id="rId4"/>
-    <sheet name="Sheet3" sheetId="14" r:id="rId5"/>
-    <sheet name="Edition" sheetId="1" r:id="rId6"/>
-    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId7"/>
-    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId8"/>
-    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId9"/>
-    <sheet name="Risk Assessment" sheetId="4" r:id="rId10"/>
-    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId11"/>
-    <sheet name="Reviewer" sheetId="6" r:id="rId12"/>
-    <sheet name="Site Visit" sheetId="5" r:id="rId13"/>
-    <sheet name="Desk Review" sheetId="7" r:id="rId14"/>
-    <sheet name="KPI" sheetId="18" r:id="rId15"/>
-    <sheet name="Sheet1" sheetId="8" r:id="rId16"/>
-    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId17"/>
-    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId18"/>
-    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId19"/>
-    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId20"/>
-    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId21"/>
-    <sheet name="Progress Report Annually" sheetId="24" r:id="rId22"/>
-    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId23"/>
-    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId24"/>
+    <sheet name="Progress Report Error" sheetId="27" r:id="rId4"/>
+    <sheet name="Grant_Edition" sheetId="11" r:id="rId5"/>
+    <sheet name="Sheet3" sheetId="14" r:id="rId6"/>
+    <sheet name="Edition" sheetId="1" r:id="rId7"/>
+    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId8"/>
+    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId9"/>
+    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId10"/>
+    <sheet name="Risk Assessment" sheetId="4" r:id="rId11"/>
+    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId12"/>
+    <sheet name="Reviewer" sheetId="6" r:id="rId13"/>
+    <sheet name="Site Visit" sheetId="5" r:id="rId14"/>
+    <sheet name="Desk Review" sheetId="7" r:id="rId15"/>
+    <sheet name="KPI" sheetId="18" r:id="rId16"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId17"/>
+    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId18"/>
+    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId19"/>
+    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId20"/>
+    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId21"/>
+    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId22"/>
+    <sheet name="Progress Report Annually" sheetId="24" r:id="rId23"/>
+    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId24"/>
+    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId25"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="118">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -798,13 +799,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -815,7 +816,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -826,7 +827,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -837,7 +838,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -848,7 +849,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -866,16 +867,108 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -886,7 +979,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -897,7 +990,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -908,7 +1001,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -919,7 +1012,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -930,7 +1023,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -941,7 +1034,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -952,7 +1045,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -963,7 +1056,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -974,7 +1067,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -985,7 +1078,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -996,7 +1089,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1007,7 +1100,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1018,7 +1111,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1029,7 +1122,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1040,7 +1133,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1051,7 +1144,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1062,7 +1155,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1073,7 +1166,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1084,7 +1177,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1100,17 +1193,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1121,7 +1214,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1138,17 +1231,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1159,7 +1252,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1170,7 +1263,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1181,7 +1274,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1192,7 +1285,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1209,16 +1302,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1229,7 +1322,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1240,7 +1333,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1251,66 +1344,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1327,15 +1361,74 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1346,7 +1439,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1357,7 +1450,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1374,21 +1467,21 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1411,7 +1504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1434,7 +1527,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1454,7 +1547,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1474,7 +1567,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1488,241 +1581,84 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>51</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>89</v>
-      </c>
-      <c r="C7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>93</v>
-      </c>
-      <c r="C11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C13" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1731,15 +1667,172 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1750,7 +1843,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1761,7 +1854,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1772,7 +1865,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1783,7 +1876,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1794,7 +1887,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1805,7 +1898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1822,108 +1915,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="18.88671875" customWidth="1"/>
-    <col min="2" max="2" width="32.6640625" customWidth="1"/>
-    <col min="3" max="3" width="49.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>3700</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1934,7 +1935,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1945,7 +1946,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1956,7 +1957,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1967,7 +1968,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1978,10 +1979,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
     </row>
@@ -1992,16 +1993,16 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" customWidth="1"/>
-    <col min="2" max="2" width="28.44140625" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" customWidth="1"/>
+    <col min="3" max="3" width="49.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2012,7 +2013,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2023,7 +2024,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2031,10 +2032,10 @@
         <v>11</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2045,7 +2046,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2056,7 +2057,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2067,7 +2068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2075,7 +2076,7 @@
         <v>101</v>
       </c>
       <c r="C7">
-        <v>365</v>
+        <v>3700</v>
       </c>
     </row>
   </sheetData>
@@ -2084,16 +2085,16 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.88671875" customWidth="1"/>
-    <col min="2" max="2" width="34.109375" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" customWidth="1"/>
+    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2104,7 +2105,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2115,7 +2116,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2123,10 +2124,10 @@
         <v>11</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2137,7 +2138,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2148,7 +2149,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2159,7 +2160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2176,15 +2177,107 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27.85546875" customWidth="1"/>
+    <col min="2" max="2" width="34.140625" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2195,7 +2288,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2206,7 +2299,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2217,7 +2310,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2228,7 +2321,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2239,7 +2332,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2250,7 +2343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2267,15 +2360,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2286,7 +2379,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2297,7 +2390,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2308,7 +2401,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2319,7 +2412,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2330,7 +2423,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2341,7 +2434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2357,15 +2450,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="24.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2376,7 +2469,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2387,7 +2480,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2398,7 +2491,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2409,7 +2502,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2420,7 +2513,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2431,7 +2524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2450,13 +2543,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
-    <col min="3" max="3" width="38.88671875" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="3" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2467,7 +2560,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2478,7 +2571,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2489,7 +2582,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2500,7 +2593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2511,7 +2604,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2522,7 +2615,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2533,7 +2626,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2544,7 +2637,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2555,7 +2648,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -2567,16 +2660,96 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5">
+        <v>-300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6">
+        <v>1000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2587,7 +2760,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2598,7 +2771,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2609,7 +2782,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2620,7 +2793,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2631,7 +2804,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2642,7 +2815,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2653,7 +2826,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2664,7 +2837,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2675,7 +2848,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2686,7 +2859,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2697,7 +2870,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2708,7 +2881,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -2725,16 +2898,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -2745,7 +2918,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2756,7 +2929,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2767,7 +2940,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -2778,7 +2951,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -2789,7 +2962,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -2800,7 +2973,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -2813,17 +2986,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2834,7 +3007,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2845,13 +3018,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C5" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
         <v>114</v>
       </c>
@@ -2862,17 +3035,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2883,7 +3056,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2894,7 +3067,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -2910,16 +3083,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2930,7 +3103,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2941,7 +3114,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2952,7 +3125,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2963,7 +3136,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2974,7 +3147,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2985,7 +3158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3000,96 +3173,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="300" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>3650</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Merged PR 2965: Merge mprod09july to master
Related work items: #55309, #57367, #57404
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91F7757-9872-4062-BB93-A5495E37EAAA}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB26E92F-03E1-4D0D-97B0-F1DCC59629E3}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="1" activeTab="3" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="8" activeTab="10" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -23,21 +23,22 @@
     <sheet name="Edition_StandAlone" sheetId="9" r:id="rId8"/>
     <sheet name="Payment Request Schedule" sheetId="2" r:id="rId9"/>
     <sheet name="Progress Report Schedule" sheetId="3" r:id="rId10"/>
-    <sheet name="Risk Assessment" sheetId="4" r:id="rId11"/>
-    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId12"/>
-    <sheet name="Reviewer" sheetId="6" r:id="rId13"/>
-    <sheet name="Site Visit" sheetId="5" r:id="rId14"/>
-    <sheet name="Desk Review" sheetId="7" r:id="rId15"/>
-    <sheet name="KPI" sheetId="18" r:id="rId16"/>
-    <sheet name="Sheet1" sheetId="8" r:id="rId17"/>
-    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId18"/>
-    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId19"/>
-    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId20"/>
-    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId21"/>
-    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId22"/>
-    <sheet name="Progress Report Annually" sheetId="24" r:id="rId23"/>
-    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId24"/>
-    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId25"/>
+    <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId11"/>
+    <sheet name="Risk Assessment" sheetId="4" r:id="rId12"/>
+    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId13"/>
+    <sheet name="Reviewer" sheetId="6" r:id="rId14"/>
+    <sheet name="Site Visit" sheetId="5" r:id="rId15"/>
+    <sheet name="Desk Review" sheetId="7" r:id="rId16"/>
+    <sheet name="KPI" sheetId="18" r:id="rId17"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId18"/>
+    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId19"/>
+    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId20"/>
+    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId21"/>
+    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId22"/>
+    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId23"/>
+    <sheet name="Progress Report Annually" sheetId="24" r:id="rId24"/>
+    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId25"/>
+    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId26"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="119">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -403,6 +404,9 @@
   </si>
   <si>
     <t>Automation Execution Award</t>
+  </si>
+  <si>
+    <t>02/02/2024</t>
   </si>
 </sst>
 </file>
@@ -467,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -484,6 +488,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -959,6 +964,97 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1193,7 +1289,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1231,7 +1327,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1302,7 +1398,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1360,7 +1456,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1419,7 +1515,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1467,7 +1563,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1666,7 +1762,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1820,98 +1916,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>3650</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1993,6 +1997,98 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2084,7 +2180,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2176,7 +2272,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2268,7 +2364,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2360,7 +2456,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2450,7 +2546,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2661,7 +2757,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
@@ -2669,25 +2765,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>9</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" t="s">
-        <v>98</v>
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2695,10 +2791,10 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2706,10 +2802,10 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2717,10 +2813,10 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C5">
-        <v>-300</v>
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2728,9 +2824,20 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>-300</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
         <v>101</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>1000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Merged PR 3018: Merge Deepika09may to master
Created and Automated 17 new test Cases in Risk Assessment Feature.
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB26E92F-03E1-4D0D-97B0-F1DCC59629E3}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08510EEC-30B3-40E2-8910-0F812096EA54}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="8" activeTab="10" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="14" activeTab="19" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -18,27 +18,30 @@
     <sheet name="Grant_Creation" sheetId="10" r:id="rId3"/>
     <sheet name="Progress Report Error" sheetId="27" r:id="rId4"/>
     <sheet name="Grant_Edition" sheetId="11" r:id="rId5"/>
-    <sheet name="Sheet3" sheetId="14" r:id="rId6"/>
-    <sheet name="Edition" sheetId="1" r:id="rId7"/>
-    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId8"/>
-    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId9"/>
-    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId10"/>
-    <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId11"/>
-    <sheet name="Risk Assessment" sheetId="4" r:id="rId12"/>
-    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId13"/>
-    <sheet name="Reviewer" sheetId="6" r:id="rId14"/>
-    <sheet name="Site Visit" sheetId="5" r:id="rId15"/>
-    <sheet name="Desk Review" sheetId="7" r:id="rId16"/>
-    <sheet name="KPI" sheetId="18" r:id="rId17"/>
-    <sheet name="Sheet1" sheetId="8" r:id="rId18"/>
-    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId19"/>
-    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId20"/>
-    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId21"/>
-    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId22"/>
-    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId23"/>
-    <sheet name="Progress Report Annually" sheetId="24" r:id="rId24"/>
-    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId25"/>
-    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId26"/>
+    <sheet name="Grant_Edition1" sheetId="30" r:id="rId6"/>
+    <sheet name="Sheet3" sheetId="14" r:id="rId7"/>
+    <sheet name="Edition" sheetId="1" r:id="rId8"/>
+    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId9"/>
+    <sheet name="Grant_Creation1" sheetId="31" r:id="rId10"/>
+    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId11"/>
+    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId12"/>
+    <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId13"/>
+    <sheet name="Risk Assessment" sheetId="4" r:id="rId14"/>
+    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId15"/>
+    <sheet name="Reviewer" sheetId="6" r:id="rId16"/>
+    <sheet name="Site Visit" sheetId="5" r:id="rId17"/>
+    <sheet name="Desk Review" sheetId="7" r:id="rId18"/>
+    <sheet name="KPI" sheetId="18" r:id="rId19"/>
+    <sheet name="Risk Assessment1" sheetId="29" r:id="rId20"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId21"/>
+    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId22"/>
+    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId23"/>
+    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId24"/>
+    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId25"/>
+    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId26"/>
+    <sheet name="Progress Report Annually" sheetId="24" r:id="rId27"/>
+    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId28"/>
+    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId29"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -50,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="120">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -403,10 +406,13 @@
     <t>z</t>
   </si>
   <si>
+    <t>02/02/2024</t>
+  </si>
+  <si>
     <t>Automation Execution Award</t>
   </si>
   <si>
-    <t>02/02/2024</t>
+    <t>Automation Award for Risk Assessment</t>
   </si>
 </sst>
 </file>
@@ -804,13 +810,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -821,7 +827,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -832,7 +838,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -843,7 +849,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -854,7 +860,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -872,15 +878,225 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G20" t="s">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -891,7 +1107,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -902,7 +1118,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -913,7 +1129,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -924,7 +1140,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -935,7 +1151,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -946,7 +1162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -963,16 +1179,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -983,7 +1199,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -994,7 +1210,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1005,7 +1221,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1016,7 +1232,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1027,7 +1243,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1035,10 +1251,10 @@
         <v>102</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1054,17 +1270,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1075,7 +1291,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1086,7 +1302,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1097,7 +1313,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1108,7 +1324,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1119,7 +1335,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1130,7 +1346,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1141,7 +1357,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1152,7 +1368,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1163,7 +1379,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1174,7 +1390,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1185,7 +1401,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1196,7 +1412,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1207,7 +1423,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1218,7 +1434,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1229,7 +1445,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1240,7 +1456,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1251,7 +1467,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1262,7 +1478,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1273,7 +1489,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1289,17 +1505,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1310,7 +1526,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1327,17 +1543,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1348,7 +1564,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1359,7 +1575,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1370,7 +1586,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1381,7 +1597,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1398,16 +1614,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1418,7 +1634,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1429,7 +1645,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1440,7 +1656,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1456,17 +1672,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1477,7 +1693,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1488,7 +1704,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1499,7 +1715,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1515,16 +1731,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1535,7 +1751,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1546,7 +1762,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1563,372 +1779,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
-  <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E17" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E18" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E19" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E20" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E21" t="s">
-        <v>51</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>89</v>
-      </c>
-      <c r="C7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>93</v>
-      </c>
-      <c r="C11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C13" t="s">
-        <v>38</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1939,7 +1799,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1950,7 +1810,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1961,7 +1821,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1972,7 +1832,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1983,10 +1843,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
     </row>
@@ -1997,15 +1857,573 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E20" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2016,7 +2434,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2027,7 +2445,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2038,7 +2456,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2049,7 +2467,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2060,7 +2478,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2071,7 +2489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2088,17 +2506,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="32.7109375" customWidth="1"/>
-    <col min="3" max="3" width="49.85546875" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="32.6640625" customWidth="1"/>
+    <col min="3" max="3" width="49.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2109,7 +2527,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2120,7 +2538,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2131,7 +2549,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2142,7 +2560,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2153,7 +2571,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2164,7 +2582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2180,17 +2598,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
-    <col min="2" max="2" width="28.42578125" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28.44140625" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2201,7 +2619,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2212,7 +2630,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2223,7 +2641,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2234,7 +2652,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2245,7 +2663,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2256,7 +2674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2272,17 +2690,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.85546875" customWidth="1"/>
-    <col min="2" max="2" width="34.140625" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="27.88671875" customWidth="1"/>
+    <col min="2" max="2" width="34.109375" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2293,7 +2711,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2304,7 +2722,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2315,7 +2733,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2326,7 +2744,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2337,7 +2755,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2348,7 +2766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2364,16 +2782,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2384,7 +2802,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2395,7 +2813,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2406,7 +2824,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2417,7 +2835,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2428,7 +2846,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2439,7 +2857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2456,15 +2874,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2475,7 +2893,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2486,7 +2904,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2497,7 +2915,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2508,7 +2926,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2519,7 +2937,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2530,7 +2948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2546,15 +2964,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2565,7 +2983,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2576,7 +2994,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2587,7 +3005,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2598,7 +3016,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2609,7 +3027,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2620,7 +3038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2639,13 +3057,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
-    <col min="3" max="3" width="38.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2656,7 +3074,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2664,10 +3082,10 @@
         <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2678,7 +3096,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2689,7 +3107,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2700,7 +3118,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2711,7 +3129,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2722,7 +3140,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2733,7 +3151,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2744,7 +3162,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -2758,13 +3176,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2775,7 +3193,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2786,7 +3204,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2797,7 +3215,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2808,7 +3226,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2819,7 +3237,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2830,7 +3248,7 @@
         <v>-300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2849,14 +3267,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2867,7 +3285,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2878,7 +3296,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2889,7 +3307,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2900,7 +3318,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2911,7 +3329,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2922,7 +3340,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2933,7 +3351,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2944,7 +3362,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2955,7 +3373,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2966,7 +3384,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2977,7 +3395,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2988,7 +3406,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3006,86 +3424,156 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2831158A-D169-49BB-9942-2243EC476E43}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>95</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>5</v>
+        <v>94</v>
       </c>
       <c r="C12" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>9</v>
-      </c>
-      <c r="B14" t="s">
-        <v>79</v>
-      </c>
-      <c r="C14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>82</v>
-      </c>
-      <c r="B16" t="s">
-        <v>83</v>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -3094,16 +3582,104 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" t="s">
+        <v>83</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3114,7 +3690,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3125,13 +3701,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C5" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
         <v>114</v>
       </c>
@@ -3142,17 +3718,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3163,7 +3739,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3174,7 +3750,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -3188,96 +3764,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>3650</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="300" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fixed Happy Path Test Cases in Amendment and Closeout Features
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB26E92F-03E1-4D0D-97B0-F1DCC59629E3}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C38CF35-3183-4A06-9D6A-43D0487DB731}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="8" activeTab="10" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -403,10 +403,10 @@
     <t>z</t>
   </si>
   <si>
+    <t>02/02/2024</t>
+  </si>
+  <si>
     <t>Automation Execution Award</t>
-  </si>
-  <si>
-    <t>02/02/2024</t>
   </si>
 </sst>
 </file>
@@ -804,13 +804,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -821,7 +821,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -832,7 +832,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -843,7 +843,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -854,7 +854,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -874,13 +874,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -891,7 +891,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -902,7 +902,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -913,7 +913,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -924,7 +924,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -935,7 +935,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -946,7 +946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -966,13 +966,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -983,7 +983,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -994,7 +994,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1035,10 +1035,10 @@
         <v>102</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1057,14 +1057,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1075,7 +1075,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1086,7 +1086,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1141,7 +1141,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1163,7 +1163,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1174,7 +1174,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1196,7 +1196,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1207,7 +1207,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1229,7 +1229,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1251,7 +1251,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1262,7 +1262,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1273,7 +1273,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1292,14 +1292,14 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1330,14 +1330,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1348,7 +1348,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1381,7 +1381,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1401,13 +1401,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1459,14 +1459,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1477,7 +1477,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1488,7 +1488,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1518,13 +1518,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1535,7 +1535,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1566,18 +1566,18 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1623,7 +1623,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1663,7 +1663,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1677,82 +1677,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -1765,13 +1765,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1782,7 +1782,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1815,7 +1815,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1848,7 +1848,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1922,13 +1922,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1939,7 +1939,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1983,10 +1983,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
     </row>
@@ -1999,13 +1999,13 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2016,7 +2016,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2027,7 +2027,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2038,7 +2038,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2049,7 +2049,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2071,7 +2071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2091,14 +2091,14 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="32.7109375" customWidth="1"/>
-    <col min="3" max="3" width="49.85546875" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="32.6640625" customWidth="1"/>
+    <col min="3" max="3" width="49.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2131,7 +2131,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2153,7 +2153,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2183,14 +2183,14 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
-    <col min="2" max="2" width="28.42578125" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28.44140625" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2201,7 +2201,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2212,7 +2212,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2223,7 +2223,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2245,7 +2245,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2256,7 +2256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2275,14 +2275,14 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.85546875" customWidth="1"/>
-    <col min="2" max="2" width="34.140625" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="27.88671875" customWidth="1"/>
+    <col min="2" max="2" width="34.109375" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2293,7 +2293,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2304,7 +2304,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2315,7 +2315,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2326,7 +2326,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2337,7 +2337,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2348,7 +2348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2367,13 +2367,13 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2384,7 +2384,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2395,7 +2395,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2417,7 +2417,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2428,7 +2428,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2439,7 +2439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2459,12 +2459,12 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2549,12 +2549,12 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2565,7 +2565,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2576,7 +2576,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2598,7 +2598,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2609,7 +2609,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2620,7 +2620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2639,13 +2639,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
-    <col min="3" max="3" width="38.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2656,7 +2656,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2664,10 +2664,10 @@
         <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2700,7 +2700,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2711,7 +2711,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -2758,13 +2758,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2775,7 +2775,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2786,7 +2786,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2797,7 +2797,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2808,7 +2808,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2830,7 +2830,7 @@
         <v>-300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2849,14 +2849,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2867,7 +2867,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2900,7 +2900,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2911,7 +2911,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2933,7 +2933,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2955,7 +2955,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2966,7 +2966,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2977,7 +2977,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2988,7 +2988,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3008,13 +3008,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -3025,7 +3025,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3036,7 +3036,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3047,7 +3047,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -3058,7 +3058,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -3069,7 +3069,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -3096,14 +3096,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3125,13 +3125,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C5" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
         <v>114</v>
       </c>
@@ -3145,14 +3145,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3163,7 +3163,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3174,7 +3174,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -3193,13 +3193,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3210,7 +3210,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3221,7 +3221,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3243,7 +3243,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 3023: Merge DeepikaRefactoringBranch to master-grey
Refactored Test Cases in Amendment and Closeout Request in test 7 from businessflow.feature
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB26E92F-03E1-4D0D-97B0-F1DCC59629E3}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C38CF35-3183-4A06-9D6A-43D0487DB731}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="8" activeTab="10" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -403,10 +403,10 @@
     <t>z</t>
   </si>
   <si>
+    <t>02/02/2024</t>
+  </si>
+  <si>
     <t>Automation Execution Award</t>
-  </si>
-  <si>
-    <t>02/02/2024</t>
   </si>
 </sst>
 </file>
@@ -804,13 +804,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -821,7 +821,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -832,7 +832,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -843,7 +843,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -854,7 +854,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -874,13 +874,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -891,7 +891,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -902,7 +902,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -913,7 +913,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -924,7 +924,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -935,7 +935,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -946,7 +946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -966,13 +966,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -983,7 +983,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -994,7 +994,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1035,10 +1035,10 @@
         <v>102</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1057,14 +1057,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1075,7 +1075,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1086,7 +1086,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1141,7 +1141,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1163,7 +1163,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1174,7 +1174,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1196,7 +1196,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1207,7 +1207,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1229,7 +1229,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1251,7 +1251,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1262,7 +1262,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1273,7 +1273,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1292,14 +1292,14 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1330,14 +1330,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1348,7 +1348,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1381,7 +1381,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1401,13 +1401,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1459,14 +1459,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1477,7 +1477,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1488,7 +1488,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1518,13 +1518,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1535,7 +1535,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1566,18 +1566,18 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1623,7 +1623,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1663,7 +1663,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1677,82 +1677,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -1765,13 +1765,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1782,7 +1782,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1815,7 +1815,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1848,7 +1848,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1922,13 +1922,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1939,7 +1939,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1983,10 +1983,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
     </row>
@@ -1999,13 +1999,13 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2016,7 +2016,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2027,7 +2027,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2038,7 +2038,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2049,7 +2049,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2071,7 +2071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2091,14 +2091,14 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="32.7109375" customWidth="1"/>
-    <col min="3" max="3" width="49.85546875" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="32.6640625" customWidth="1"/>
+    <col min="3" max="3" width="49.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2131,7 +2131,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2153,7 +2153,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2183,14 +2183,14 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
-    <col min="2" max="2" width="28.42578125" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28.44140625" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2201,7 +2201,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2212,7 +2212,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2223,7 +2223,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2245,7 +2245,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2256,7 +2256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2275,14 +2275,14 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.85546875" customWidth="1"/>
-    <col min="2" max="2" width="34.140625" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="27.88671875" customWidth="1"/>
+    <col min="2" max="2" width="34.109375" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2293,7 +2293,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2304,7 +2304,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2315,7 +2315,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2326,7 +2326,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2337,7 +2337,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2348,7 +2348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2367,13 +2367,13 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2384,7 +2384,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2395,7 +2395,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2417,7 +2417,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2428,7 +2428,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2439,7 +2439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2459,12 +2459,12 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2549,12 +2549,12 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2565,7 +2565,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2576,7 +2576,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2598,7 +2598,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2609,7 +2609,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2620,7 +2620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2639,13 +2639,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
-    <col min="3" max="3" width="38.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2656,7 +2656,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2664,10 +2664,10 @@
         <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2700,7 +2700,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2711,7 +2711,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -2758,13 +2758,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2775,7 +2775,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2786,7 +2786,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2797,7 +2797,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2808,7 +2808,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2830,7 +2830,7 @@
         <v>-300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2849,14 +2849,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2867,7 +2867,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2900,7 +2900,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2911,7 +2911,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2933,7 +2933,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2955,7 +2955,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2966,7 +2966,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2977,7 +2977,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2988,7 +2988,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3008,13 +3008,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -3025,7 +3025,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3036,7 +3036,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3047,7 +3047,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -3058,7 +3058,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -3069,7 +3069,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -3096,14 +3096,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3125,13 +3125,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C5" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
         <v>114</v>
       </c>
@@ -3145,14 +3145,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3163,7 +3163,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3174,7 +3174,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -3193,13 +3193,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3210,7 +3210,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3221,7 +3221,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3243,7 +3243,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 3062: Merge m19julyqafix to master-grey
refactored test cases on QA
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB1336D-34F0-4B4D-AF77-20F520176418}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08510EEC-30B3-40E2-8910-0F812096EA54}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="14" activeTab="19" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -18,27 +18,30 @@
     <sheet name="Grant_Creation" sheetId="10" r:id="rId3"/>
     <sheet name="Progress Report Error" sheetId="27" r:id="rId4"/>
     <sheet name="Grant_Edition" sheetId="11" r:id="rId5"/>
-    <sheet name="Sheet3" sheetId="14" r:id="rId6"/>
-    <sheet name="Edition" sheetId="1" r:id="rId7"/>
-    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId8"/>
-    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId9"/>
-    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId10"/>
-    <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId11"/>
-    <sheet name="Risk Assessment" sheetId="4" r:id="rId12"/>
-    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId13"/>
-    <sheet name="Reviewer" sheetId="6" r:id="rId14"/>
-    <sheet name="Site Visit" sheetId="5" r:id="rId15"/>
-    <sheet name="Desk Review" sheetId="7" r:id="rId16"/>
-    <sheet name="KPI" sheetId="18" r:id="rId17"/>
-    <sheet name="Sheet1" sheetId="8" r:id="rId18"/>
-    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId19"/>
-    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId20"/>
-    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId21"/>
-    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId22"/>
-    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId23"/>
-    <sheet name="Progress Report Annually" sheetId="24" r:id="rId24"/>
-    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId25"/>
-    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId26"/>
+    <sheet name="Grant_Edition1" sheetId="30" r:id="rId6"/>
+    <sheet name="Sheet3" sheetId="14" r:id="rId7"/>
+    <sheet name="Edition" sheetId="1" r:id="rId8"/>
+    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId9"/>
+    <sheet name="Grant_Creation1" sheetId="31" r:id="rId10"/>
+    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId11"/>
+    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId12"/>
+    <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId13"/>
+    <sheet name="Risk Assessment" sheetId="4" r:id="rId14"/>
+    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId15"/>
+    <sheet name="Reviewer" sheetId="6" r:id="rId16"/>
+    <sheet name="Site Visit" sheetId="5" r:id="rId17"/>
+    <sheet name="Desk Review" sheetId="7" r:id="rId18"/>
+    <sheet name="KPI" sheetId="18" r:id="rId19"/>
+    <sheet name="Risk Assessment1" sheetId="29" r:id="rId20"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId21"/>
+    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId22"/>
+    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId23"/>
+    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId24"/>
+    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId25"/>
+    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId26"/>
+    <sheet name="Progress Report Annually" sheetId="24" r:id="rId27"/>
+    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId28"/>
+    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId29"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -50,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="120">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -407,6 +410,9 @@
   </si>
   <si>
     <t>Automation Execution Award</t>
+  </si>
+  <si>
+    <t>Automation Award for Risk Assessment</t>
   </si>
 </sst>
 </file>
@@ -872,6 +878,216 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G20" t="s">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -963,7 +1179,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1054,7 +1270,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1289,7 +1505,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1327,7 +1543,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1398,7 +1614,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1456,7 +1672,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1515,7 +1731,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1563,7 +1779,286 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B7" s="3"/>
+      <c r="C7" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1762,7 +2257,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1919,84 +2414,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="3"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B7" s="3"/>
-      <c r="C7" s="4"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="300" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2088,7 +2506,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2180,7 +2598,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2272,7 +2690,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2364,7 +2782,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2456,7 +2874,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2546,7 +2964,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3006,6 +3424,164 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2831158A-D169-49BB-9942-2243EC476E43}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3093,7 +3669,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3142,7 +3718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3188,96 +3764,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>3650</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="300" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Merged PR 3096: Merge m21july to master-grey
Added new test cases and updated existing
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Grey\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08510EEC-30B3-40E2-8910-0F812096EA54}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0685B2B-C7E1-4AC3-95AD-E9208A50A99E}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="14" activeTab="19" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="30" activeTab="31" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -42,6 +42,9 @@
     <sheet name="Progress Report Annually" sheetId="24" r:id="rId27"/>
     <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId28"/>
     <sheet name="Progress Report Monthly" sheetId="26" r:id="rId29"/>
+    <sheet name="Progress Report StartDate Error" sheetId="32" r:id="rId30"/>
+    <sheet name="Progress Report MoreThanOneyear" sheetId="33" r:id="rId31"/>
+    <sheet name="ProgressReportQuartelyReporting" sheetId="34" r:id="rId32"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -53,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="120">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -810,13 +813,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -827,7 +830,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -838,7 +841,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -849,7 +852,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -860,7 +863,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -880,13 +883,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
-    <col min="3" max="3" width="38.88671875" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="3" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -897,7 +900,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -908,7 +911,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -919,7 +922,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -930,7 +933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -941,7 +944,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -952,7 +955,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -963,7 +966,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -974,7 +977,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -985,7 +988,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -998,13 +1001,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1015,7 +1018,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1026,7 +1029,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1037,7 +1040,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1048,7 +1051,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1059,7 +1062,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1070,7 +1073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1090,13 +1093,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1107,7 +1110,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1118,7 +1121,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1129,7 +1132,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1140,7 +1143,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1151,7 +1154,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1162,7 +1165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1182,13 +1185,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1199,7 +1202,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1210,7 +1213,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1221,7 +1224,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1232,7 +1235,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1243,7 +1246,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1254,7 +1257,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1273,14 +1276,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1291,7 +1294,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1302,7 +1305,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1313,7 +1316,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1324,7 +1327,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1335,7 +1338,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1346,7 +1349,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1357,7 +1360,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1368,7 +1371,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1379,7 +1382,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1390,7 +1393,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1401,7 +1404,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1412,7 +1415,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1423,7 +1426,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1434,7 +1437,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1445,7 +1448,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1456,7 +1459,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1467,7 +1470,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1478,7 +1481,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1489,7 +1492,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1508,14 +1511,14 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1526,7 +1529,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1546,14 +1549,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1564,7 +1567,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1575,7 +1578,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1586,7 +1589,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1597,7 +1600,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1617,13 +1620,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1634,7 +1637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1645,7 +1648,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1656,7 +1659,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1675,14 +1678,14 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1693,7 +1696,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1704,7 +1707,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1715,7 +1718,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1734,13 +1737,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1751,7 +1754,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1762,7 +1765,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1782,13 +1785,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1799,7 +1802,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1810,7 +1813,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1821,7 +1824,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1832,7 +1835,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1843,10 +1846,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
     </row>
@@ -1859,14 +1862,14 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1877,7 +1880,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1888,7 +1891,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1899,7 +1902,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1910,7 +1913,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1921,7 +1924,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1932,7 +1935,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1943,7 +1946,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1954,7 +1957,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1965,7 +1968,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1976,7 +1979,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1987,7 +1990,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1998,7 +2001,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -2009,7 +2012,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -2020,7 +2023,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -2031,7 +2034,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -2042,7 +2045,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -2061,18 +2064,18 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2095,7 +2098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -2118,7 +2121,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -2138,7 +2141,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -2158,7 +2161,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -2172,82 +2175,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -2260,13 +2263,13 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2277,7 +2280,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2288,7 +2291,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2299,7 +2302,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2310,7 +2313,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2321,7 +2324,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2332,7 +2335,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2343,7 +2346,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2354,7 +2357,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2365,7 +2368,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2376,7 +2379,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2387,7 +2390,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2398,7 +2401,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -2417,13 +2420,13 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2434,7 +2437,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2445,7 +2448,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2456,7 +2459,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2467,7 +2470,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2478,7 +2481,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2489,7 +2492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2509,14 +2512,14 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" customWidth="1"/>
-    <col min="2" max="2" width="32.6640625" customWidth="1"/>
-    <col min="3" max="3" width="49.88671875" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" customWidth="1"/>
+    <col min="3" max="3" width="49.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2527,7 +2530,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2538,7 +2541,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2549,7 +2552,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2560,7 +2563,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2571,7 +2574,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2582,7 +2585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2601,14 +2604,14 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" customWidth="1"/>
-    <col min="2" max="2" width="28.44140625" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" customWidth="1"/>
+    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2619,7 +2622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2630,7 +2633,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2641,7 +2644,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2652,7 +2655,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2663,7 +2666,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2674,7 +2677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2693,14 +2696,14 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.88671875" customWidth="1"/>
-    <col min="2" max="2" width="34.109375" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" customWidth="1"/>
+    <col min="2" max="2" width="34.140625" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2711,7 +2714,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2722,7 +2725,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2733,7 +2736,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2744,7 +2747,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2755,7 +2758,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2766,7 +2769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2785,13 +2788,13 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2802,7 +2805,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2813,7 +2816,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2824,7 +2827,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2835,7 +2838,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2846,7 +2849,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2857,7 +2860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2877,12 +2880,12 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2893,7 +2896,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2904,7 +2907,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2915,7 +2918,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2926,7 +2929,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2937,7 +2940,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2948,7 +2951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2967,12 +2970,13 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2983,7 +2987,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2994,7 +2998,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3005,7 +3009,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3016,7 +3020,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3027,7 +3031,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3038,7 +3042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3057,13 +3061,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
-    <col min="3" max="3" width="38.88671875" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="3" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3074,7 +3078,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3085,7 +3089,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3096,7 +3100,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3107,7 +3111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3118,7 +3122,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3129,7 +3133,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3140,7 +3144,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3151,7 +3155,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3162,7 +3166,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -3173,16 +3177,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3193,7 +3197,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3204,18 +3208,291 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
+      <c r="C3" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F3B454-4DBA-4E9B-A949-C34CD2C245D5}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>480</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268CDBE-0606-4B65-A8F6-04136D2C40DC}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>460</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
       <c r="C3" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3226,7 +3503,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3237,7 +3514,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3248,7 +3525,7 @@
         <v>-300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3267,14 +3544,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3285,7 +3562,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3296,7 +3573,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3307,7 +3584,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3318,7 +3595,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3329,7 +3606,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3340,7 +3617,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3351,7 +3628,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3362,7 +3639,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3373,7 +3650,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3384,7 +3661,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3395,7 +3672,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3406,7 +3683,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3426,14 +3703,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2831158A-D169-49BB-9942-2243EC476E43}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3444,7 +3721,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3455,7 +3732,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3466,7 +3743,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3477,7 +3754,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3488,7 +3765,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3499,7 +3776,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3510,7 +3787,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3521,7 +3798,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3532,7 +3809,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3543,7 +3820,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3554,7 +3831,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3565,7 +3842,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3584,13 +3861,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -3601,7 +3878,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3612,7 +3889,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3623,7 +3900,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -3634,7 +3911,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -3645,7 +3922,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -3656,7 +3933,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -3672,14 +3949,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3690,7 +3967,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3701,13 +3978,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C5" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
         <v>114</v>
       </c>
@@ -3721,14 +3998,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3739,7 +4016,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3750,7 +4027,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 3102: Merge DeepikaRefactoringGrey to master-grey
Refactored test cases
Created a new step
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Grey\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0685B2B-C7E1-4AC3-95AD-E9208A50A99E}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E39085B1-2016-44C0-AE1A-D38D4609EA6D}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="30" activeTab="31" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="2" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -412,10 +412,10 @@
     <t>02/02/2024</t>
   </si>
   <si>
-    <t>Automation Execution Award</t>
-  </si>
-  <si>
     <t>Automation Award for Risk Assessment</t>
+  </si>
+  <si>
+    <t>Automation Execution Award </t>
   </si>
 </sst>
 </file>
@@ -813,13 +813,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -830,7 +830,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -841,7 +841,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -852,7 +852,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -863,7 +863,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -883,13 +883,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
-    <col min="3" max="3" width="38.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -900,7 +900,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -908,10 +908,10 @@
         <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -922,7 +922,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -933,7 +933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -944,7 +944,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -955,7 +955,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -966,7 +966,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -977,7 +977,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -988,7 +988,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -1001,13 +1001,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1018,7 +1018,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1029,7 +1029,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1040,7 +1040,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1051,7 +1051,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1093,13 +1093,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1110,7 +1110,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1132,7 +1132,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1154,7 +1154,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1165,7 +1165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1185,13 +1185,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1224,7 +1224,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1276,14 +1276,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1294,7 +1294,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1316,7 +1316,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1327,7 +1327,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1338,7 +1338,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1349,7 +1349,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1360,7 +1360,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1371,7 +1371,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1382,7 +1382,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1404,7 +1404,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1437,7 +1437,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1481,7 +1481,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1492,7 +1492,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1511,14 +1511,14 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1549,14 +1549,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1567,7 +1567,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1578,7 +1578,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1589,7 +1589,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1620,13 +1620,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1637,7 +1637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1659,7 +1659,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1678,14 +1678,14 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1707,7 +1707,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1718,7 +1718,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1737,13 +1737,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1754,7 +1754,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1765,7 +1765,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1785,13 +1785,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1802,7 +1802,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1813,7 +1813,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1846,10 +1846,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
     </row>
@@ -1862,14 +1862,14 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1990,7 +1990,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -2001,7 +2001,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -2012,7 +2012,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -2034,7 +2034,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -2045,7 +2045,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -2064,18 +2064,18 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -2121,7 +2121,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -2161,7 +2161,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -2175,82 +2175,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -2263,13 +2263,13 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2401,7 +2401,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -2420,13 +2420,13 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2437,7 +2437,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2448,7 +2448,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2470,7 +2470,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2481,7 +2481,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2492,7 +2492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2512,14 +2512,14 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="32.7109375" customWidth="1"/>
-    <col min="3" max="3" width="49.85546875" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="32.6640625" customWidth="1"/>
+    <col min="3" max="3" width="49.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2541,7 +2541,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2604,14 +2604,14 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
-    <col min="2" max="2" width="28.42578125" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28.44140625" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2622,7 +2622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2633,7 +2633,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2655,7 +2655,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2666,7 +2666,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2677,7 +2677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2696,14 +2696,14 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.85546875" customWidth="1"/>
-    <col min="2" max="2" width="34.140625" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="27.88671875" customWidth="1"/>
+    <col min="2" max="2" width="34.109375" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2714,7 +2714,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2725,7 +2725,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2736,7 +2736,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2747,7 +2747,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2758,7 +2758,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2769,7 +2769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2788,13 +2788,13 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2827,7 +2827,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2838,7 +2838,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2860,7 +2860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2880,12 +2880,12 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2907,7 +2907,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2918,7 +2918,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2940,7 +2940,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2951,7 +2951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2970,13 +2970,13 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2987,7 +2987,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2998,7 +2998,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3009,7 +3009,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3020,7 +3020,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3031,7 +3031,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3061,13 +3061,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
-    <col min="3" max="3" width="38.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3078,7 +3078,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3086,10 +3086,10 @@
         <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3100,7 +3100,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3111,7 +3111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3122,7 +3122,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3133,7 +3133,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3155,7 +3155,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3166,7 +3166,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -3180,13 +3180,13 @@
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3197,7 +3197,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3219,7 +3219,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3252,7 +3252,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3271,13 +3271,13 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F3B454-4DBA-4E9B-A949-C34CD2C245D5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3288,7 +3288,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3299,7 +3299,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3321,7 +3321,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3332,7 +3332,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3343,7 +3343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3362,13 +3362,13 @@
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268CDBE-0606-4B65-A8F6-04136D2C40DC}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3401,7 +3401,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3453,13 +3453,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3470,7 +3470,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3481,7 +3481,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3492,7 +3492,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3503,7 +3503,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3525,7 +3525,7 @@
         <v>-300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3544,14 +3544,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3562,7 +3562,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3595,7 +3595,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3606,7 +3606,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3617,7 +3617,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3628,7 +3628,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3650,7 +3650,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3661,7 +3661,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3672,7 +3672,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3683,7 +3683,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3703,14 +3703,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2831158A-D169-49BB-9942-2243EC476E43}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3721,7 +3721,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3732,7 +3732,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3743,7 +3743,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3754,7 +3754,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3765,7 +3765,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3776,7 +3776,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3787,7 +3787,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3809,7 +3809,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3820,7 +3820,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3831,7 +3831,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3842,7 +3842,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3861,13 +3861,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -3878,7 +3878,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3889,7 +3889,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3900,7 +3900,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -3911,7 +3911,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -3922,7 +3922,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -3933,7 +3933,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -3949,14 +3949,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3967,7 +3967,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3978,13 +3978,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C5" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
         <v>114</v>
       </c>
@@ -3998,14 +3998,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4016,7 +4016,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -4027,7 +4027,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>81</v>
       </c>

</xml_diff>

<commit_message>
created new excel file for error related test cases and removed extra spaces from the existing excel sheet
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E39085B1-2016-44C0-AE1A-D38D4609EA6D}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0C4DA5A-5394-40D6-8125-775AB089EC87}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="2" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" firstSheet="2" activeTab="2" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -415,7 +415,7 @@
     <t>Automation Award for Risk Assessment</t>
   </si>
   <si>
-    <t>Automation Execution Award </t>
+    <t>Automation Execution Award</t>
   </si>
 </sst>
 </file>
@@ -813,13 +813,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -830,7 +830,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -841,7 +841,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -852,7 +852,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -863,7 +863,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -883,13 +883,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
-    <col min="3" max="3" width="38.88671875" customWidth="1"/>
+    <col min="2" max="2" width="26.07421875" customWidth="1"/>
+    <col min="3" max="3" width="38.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -900,7 +900,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -911,7 +911,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -922,7 +922,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -933,7 +933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -944,7 +944,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -955,7 +955,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -966,7 +966,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -977,7 +977,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -988,7 +988,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -1001,13 +1001,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1018,7 +1018,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1029,7 +1029,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1040,7 +1040,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1051,7 +1051,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1093,13 +1093,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1110,7 +1110,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1132,7 +1132,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1154,7 +1154,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1165,7 +1165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1185,13 +1185,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1224,7 +1224,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1276,14 +1276,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1294,7 +1294,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1316,7 +1316,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1327,7 +1327,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1338,7 +1338,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1349,7 +1349,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1360,7 +1360,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1371,7 +1371,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1382,7 +1382,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1404,7 +1404,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1437,7 +1437,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1481,7 +1481,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1492,7 +1492,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1511,14 +1511,14 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.07421875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.4609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1549,14 +1549,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1567,7 +1567,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1578,7 +1578,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1589,7 +1589,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1620,13 +1620,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.4609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1637,7 +1637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1659,7 +1659,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1678,14 +1678,14 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1707,7 +1707,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1718,7 +1718,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1737,13 +1737,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" customWidth="1"/>
+    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.07421875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1754,7 +1754,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1765,7 +1765,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1785,13 +1785,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1802,7 +1802,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1813,7 +1813,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1846,10 +1846,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
     </row>
@@ -1862,14 +1862,14 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1990,7 +1990,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -2001,7 +2001,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -2012,7 +2012,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -2034,7 +2034,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -2045,7 +2045,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -2064,18 +2064,18 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.4609375" customWidth="1"/>
+    <col min="2" max="2" width="9.69140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="4" max="4" width="10.3046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.07421875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.4609375" customWidth="1"/>
+    <col min="7" max="7" width="13.4609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -2121,7 +2121,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -2161,7 +2161,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -2175,82 +2175,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -2263,13 +2263,13 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.84375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2401,7 +2401,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -2420,13 +2420,13 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2437,7 +2437,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2448,7 +2448,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2470,7 +2470,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2481,7 +2481,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2492,7 +2492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2512,14 +2512,14 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" customWidth="1"/>
-    <col min="2" max="2" width="32.6640625" customWidth="1"/>
-    <col min="3" max="3" width="49.88671875" customWidth="1"/>
+    <col min="1" max="1" width="18.84375" customWidth="1"/>
+    <col min="2" max="2" width="32.69140625" customWidth="1"/>
+    <col min="3" max="3" width="49.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2541,7 +2541,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2604,14 +2604,14 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" customWidth="1"/>
-    <col min="2" max="2" width="28.44140625" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" customWidth="1"/>
+    <col min="1" max="1" width="24.69140625" customWidth="1"/>
+    <col min="2" max="2" width="28.4609375" customWidth="1"/>
+    <col min="3" max="3" width="29.3046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2622,7 +2622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2633,7 +2633,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2655,7 +2655,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2666,7 +2666,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2677,7 +2677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2696,14 +2696,14 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="27.88671875" customWidth="1"/>
-    <col min="2" max="2" width="34.109375" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" customWidth="1"/>
+    <col min="1" max="1" width="27.84375" customWidth="1"/>
+    <col min="2" max="2" width="34.07421875" customWidth="1"/>
+    <col min="3" max="3" width="29.3046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2714,7 +2714,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2725,7 +2725,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2736,7 +2736,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2747,7 +2747,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2758,7 +2758,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2769,7 +2769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2788,13 +2788,13 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2827,7 +2827,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2838,7 +2838,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2860,7 +2860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2880,12 +2880,12 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2907,7 +2907,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2918,7 +2918,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2940,7 +2940,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2951,7 +2951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2970,13 +2970,13 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="11.88671875" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.84375" customWidth="1"/>
+    <col min="3" max="3" width="24.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2987,7 +2987,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2998,7 +2998,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3009,7 +3009,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3020,7 +3020,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3031,7 +3031,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3061,13 +3061,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
-    <col min="3" max="3" width="38.88671875" customWidth="1"/>
+    <col min="2" max="2" width="26.07421875" customWidth="1"/>
+    <col min="3" max="3" width="38.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3078,7 +3078,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3100,7 +3100,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3111,7 +3111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3122,7 +3122,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3133,7 +3133,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3155,7 +3155,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3166,7 +3166,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.4">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -3180,13 +3180,13 @@
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3197,7 +3197,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3219,7 +3219,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3252,7 +3252,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3271,13 +3271,13 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F3B454-4DBA-4E9B-A949-C34CD2C245D5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3288,7 +3288,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3299,7 +3299,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3321,7 +3321,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3332,7 +3332,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3343,7 +3343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3362,13 +3362,13 @@
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268CDBE-0606-4B65-A8F6-04136D2C40DC}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3401,7 +3401,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3453,13 +3453,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3470,7 +3470,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3481,7 +3481,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3492,7 +3492,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3503,7 +3503,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3525,7 +3525,7 @@
         <v>-300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3544,14 +3544,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.69140625" customWidth="1"/>
+    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3562,7 +3562,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3595,7 +3595,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3606,7 +3606,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3617,7 +3617,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3628,7 +3628,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3650,7 +3650,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3661,7 +3661,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3672,7 +3672,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3683,7 +3683,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3703,14 +3703,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2831158A-D169-49BB-9942-2243EC476E43}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.69140625" customWidth="1"/>
+    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3721,7 +3721,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3732,7 +3732,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3743,7 +3743,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3754,7 +3754,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3765,7 +3765,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3776,7 +3776,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3787,7 +3787,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3809,7 +3809,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3820,7 +3820,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3831,7 +3831,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3842,7 +3842,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3861,13 +3861,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.07421875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -3878,7 +3878,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3889,7 +3889,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3900,7 +3900,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -3911,7 +3911,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -3922,7 +3922,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -3933,7 +3933,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -3949,14 +3949,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.69140625" customWidth="1"/>
+    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3967,7 +3967,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3978,13 +3978,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="C5" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="D7" t="s">
         <v>114</v>
       </c>
@@ -3998,14 +3998,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.69140625" customWidth="1"/>
+    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4016,7 +4016,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -4027,7 +4027,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>81</v>
       </c>

</xml_diff>

<commit_message>
Added new test cases and steps
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Product Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0C4DA5A-5394-40D6-8125-775AB089EC87}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D132C47A-A25C-4B2F-BE62-D7750971C12E}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" firstSheet="2" activeTab="2" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="13" activeTab="17" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="122">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -416,6 +416,12 @@
   </si>
   <si>
     <t>Automation Execution Award</t>
+  </si>
+  <si>
+    <t>Automation Progress Report</t>
+  </si>
+  <si>
+    <t>Automation Payment Request</t>
   </si>
 </sst>
 </file>
@@ -813,13 +819,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -830,7 +836,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -841,7 +847,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -852,7 +858,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -863,7 +869,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -883,13 +889,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.07421875" customWidth="1"/>
-    <col min="3" max="3" width="38.84375" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="3" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -900,7 +906,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -911,7 +917,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -922,7 +928,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -933,7 +939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -944,7 +950,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -955,7 +961,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -966,7 +972,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -977,7 +983,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -988,7 +994,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -1001,13 +1007,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1018,7 +1024,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1026,10 +1032,10 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1040,7 +1046,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1051,7 +1057,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1062,7 +1068,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1073,7 +1079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1093,13 +1099,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1110,7 +1116,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1118,10 +1124,10 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1132,7 +1138,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1143,7 +1149,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1154,7 +1160,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1165,7 +1171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1185,13 +1191,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1202,7 +1208,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1213,7 +1219,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1224,7 +1230,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1235,7 +1241,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1246,7 +1252,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1257,7 +1263,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1276,14 +1282,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1294,7 +1300,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1305,7 +1311,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1316,7 +1322,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1327,7 +1333,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1338,7 +1344,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1349,7 +1355,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1360,7 +1366,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1371,7 +1377,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1382,7 +1388,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1393,7 +1399,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1404,7 +1410,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1415,7 +1421,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1426,7 +1432,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1437,7 +1443,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1448,7 +1454,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1459,7 +1465,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1470,7 +1476,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1481,7 +1487,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1492,7 +1498,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1511,14 +1517,14 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.4609375" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1529,7 +1535,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1549,14 +1555,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1567,7 +1573,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1578,7 +1584,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1589,7 +1595,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1600,7 +1606,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1620,13 +1626,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.4609375" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1637,7 +1643,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1648,7 +1654,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1659,7 +1665,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1678,14 +1684,14 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1696,7 +1702,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1707,7 +1713,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1718,7 +1724,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1737,13 +1743,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.07421875" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1754,7 +1760,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1765,7 +1771,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1785,13 +1791,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1802,7 +1808,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1813,7 +1819,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1824,7 +1830,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1835,7 +1841,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1846,10 +1852,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
     </row>
@@ -1862,14 +1868,14 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1880,7 +1886,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1891,7 +1897,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1902,7 +1908,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1913,7 +1919,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1924,7 +1930,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1935,7 +1941,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1946,7 +1952,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1957,7 +1963,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1968,7 +1974,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1979,7 +1985,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1990,7 +1996,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -2001,7 +2007,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -2012,7 +2018,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -2023,7 +2029,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -2034,7 +2040,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -2045,7 +2051,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -2064,18 +2070,18 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.4609375" customWidth="1"/>
-    <col min="2" max="2" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.3046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.07421875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.4609375" customWidth="1"/>
-    <col min="7" max="7" width="13.4609375" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2098,7 +2104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -2121,7 +2127,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -2141,7 +2147,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -2161,7 +2167,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -2175,82 +2181,82 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
         <v>51</v>
       </c>
@@ -2263,13 +2269,13 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.84375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2280,7 +2286,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2291,7 +2297,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2302,7 +2308,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2313,7 +2319,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2324,7 +2330,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2335,7 +2341,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2346,7 +2352,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2357,7 +2363,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2368,7 +2374,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2379,7 +2385,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2390,7 +2396,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2401,7 +2407,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -2420,13 +2426,13 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2437,7 +2443,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2448,7 +2454,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2459,7 +2465,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2470,7 +2476,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2481,7 +2487,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2492,7 +2498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2512,14 +2518,14 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.84375" customWidth="1"/>
-    <col min="2" max="2" width="32.69140625" customWidth="1"/>
-    <col min="3" max="3" width="49.84375" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" customWidth="1"/>
+    <col min="3" max="3" width="49.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2530,7 +2536,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2541,7 +2547,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2552,7 +2558,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2563,7 +2569,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2574,7 +2580,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2585,7 +2591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2604,14 +2610,14 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.69140625" customWidth="1"/>
-    <col min="2" max="2" width="28.4609375" customWidth="1"/>
-    <col min="3" max="3" width="29.3046875" customWidth="1"/>
+    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2622,7 +2628,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2633,7 +2639,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2644,7 +2650,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2655,7 +2661,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2666,7 +2672,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2677,7 +2683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2696,14 +2702,14 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.84375" customWidth="1"/>
-    <col min="2" max="2" width="34.07421875" customWidth="1"/>
-    <col min="3" max="3" width="29.3046875" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" customWidth="1"/>
+    <col min="2" max="2" width="34.140625" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2714,7 +2720,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2725,7 +2731,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2736,7 +2742,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2747,7 +2753,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2758,7 +2764,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2769,7 +2775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2788,13 +2794,13 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2805,7 +2811,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2816,7 +2822,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2827,7 +2833,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2838,7 +2844,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2849,7 +2855,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2860,7 +2866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2880,12 +2886,12 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2896,7 +2902,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2907,7 +2913,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2918,7 +2924,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2929,7 +2935,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2940,7 +2946,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2951,7 +2957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2970,13 +2976,13 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.84375" customWidth="1"/>
-    <col min="3" max="3" width="24.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2987,7 +2993,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2998,7 +3004,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3009,7 +3015,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3020,7 +3026,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3031,7 +3037,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3042,7 +3048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3061,13 +3067,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.07421875" customWidth="1"/>
-    <col min="3" max="3" width="38.84375" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="3" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3078,7 +3084,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3089,7 +3095,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3100,7 +3106,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3111,7 +3117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3122,7 +3128,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3133,7 +3139,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3144,7 +3150,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3155,7 +3161,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3166,7 +3172,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -3180,13 +3186,13 @@
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3197,7 +3203,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3208,7 +3214,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3219,7 +3225,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3230,7 +3236,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3241,7 +3247,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3252,7 +3258,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3271,13 +3277,13 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F3B454-4DBA-4E9B-A949-C34CD2C245D5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3288,7 +3294,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3299,7 +3305,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3310,7 +3316,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3321,7 +3327,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3332,7 +3338,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3343,7 +3349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3362,13 +3368,13 @@
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268CDBE-0606-4B65-A8F6-04136D2C40DC}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3379,7 +3385,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3390,7 +3396,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3401,7 +3407,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3412,7 +3418,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3423,7 +3429,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3434,7 +3440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3453,13 +3459,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3470,7 +3476,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3478,10 +3484,10 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3492,7 +3498,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3503,7 +3509,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3514,7 +3520,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3525,7 +3531,7 @@
         <v>-300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3544,14 +3550,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.69140625" customWidth="1"/>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3562,7 +3568,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3573,7 +3579,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3584,7 +3590,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3595,7 +3601,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3606,7 +3612,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3617,7 +3623,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3628,7 +3634,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3639,7 +3645,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3650,7 +3656,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3661,7 +3667,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3672,7 +3678,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3683,7 +3689,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3703,14 +3709,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2831158A-D169-49BB-9942-2243EC476E43}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.69140625" customWidth="1"/>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3721,7 +3727,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3732,7 +3738,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3743,7 +3749,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3754,7 +3760,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3765,7 +3771,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3776,7 +3782,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3787,7 +3793,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3798,7 +3804,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3809,7 +3815,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3820,7 +3826,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3831,7 +3837,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3842,7 +3848,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3861,13 +3867,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.53515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -3878,7 +3884,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3889,7 +3895,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3900,7 +3906,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -3911,7 +3917,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -3922,7 +3928,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -3933,7 +3939,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -3949,14 +3955,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3967,7 +3973,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3978,13 +3984,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C5" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
         <v>114</v>
       </c>
@@ -3998,14 +4004,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4016,7 +4022,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -4027,7 +4033,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>

</xml_diff>

<commit_message>
add new test cases and refactored test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0C4DA5A-5394-40D6-8125-775AB089EC87}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6941E37-613D-4157-A9D9-D679CD10CF64}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" firstSheet="2" activeTab="2" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="12" activeTab="15" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -28,23 +28,25 @@
     <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId13"/>
     <sheet name="Risk Assessment" sheetId="4" r:id="rId14"/>
     <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId15"/>
-    <sheet name="Reviewer" sheetId="6" r:id="rId16"/>
-    <sheet name="Site Visit" sheetId="5" r:id="rId17"/>
-    <sheet name="Desk Review" sheetId="7" r:id="rId18"/>
-    <sheet name="KPI" sheetId="18" r:id="rId19"/>
-    <sheet name="Risk Assessment1" sheetId="29" r:id="rId20"/>
-    <sheet name="Sheet1" sheetId="8" r:id="rId21"/>
-    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId22"/>
-    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId23"/>
-    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId24"/>
-    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId25"/>
-    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId26"/>
-    <sheet name="Progress Report Annually" sheetId="24" r:id="rId27"/>
-    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId28"/>
-    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId29"/>
-    <sheet name="Progress Report StartDate Error" sheetId="32" r:id="rId30"/>
-    <sheet name="Progress Report MoreThanOneyear" sheetId="33" r:id="rId31"/>
-    <sheet name="ProgressReportQuartelyReporting" sheetId="34" r:id="rId32"/>
+    <sheet name="Risk Assessment RA1" sheetId="36" r:id="rId16"/>
+    <sheet name="Risk Assessment Creation1" sheetId="35" r:id="rId17"/>
+    <sheet name="Reviewer" sheetId="6" r:id="rId18"/>
+    <sheet name="Site Visit" sheetId="5" r:id="rId19"/>
+    <sheet name="Desk Review" sheetId="7" r:id="rId20"/>
+    <sheet name="KPI" sheetId="18" r:id="rId21"/>
+    <sheet name="Risk Assessment1" sheetId="29" r:id="rId22"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId23"/>
+    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId24"/>
+    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId25"/>
+    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId26"/>
+    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId27"/>
+    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId28"/>
+    <sheet name="Progress Report Annually" sheetId="24" r:id="rId29"/>
+    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId30"/>
+    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId31"/>
+    <sheet name="Progress Report StartDate Error" sheetId="32" r:id="rId32"/>
+    <sheet name="Progress Report MoreThanOneyear" sheetId="33" r:id="rId33"/>
+    <sheet name="ProgressReportQuartelyReporting" sheetId="34" r:id="rId34"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -56,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="126">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -416,6 +418,24 @@
   </si>
   <si>
     <t>Automation Execution Award</t>
+  </si>
+  <si>
+    <t>Always</t>
+  </si>
+  <si>
+    <t>Yes, in  the last two years</t>
+  </si>
+  <si>
+    <t>Not Applicable - N/A</t>
+  </si>
+  <si>
+    <t>Rarely</t>
+  </si>
+  <si>
+    <t>1-3 years</t>
+  </si>
+  <si>
+    <t>No findings</t>
   </si>
 </sst>
 </file>
@@ -813,13 +833,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -830,7 +850,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -841,7 +861,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -852,7 +872,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -863,7 +883,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -883,13 +903,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.07421875" customWidth="1"/>
-    <col min="3" max="3" width="38.84375" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -900,7 +920,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -911,7 +931,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -922,7 +942,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -933,7 +953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -944,7 +964,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -955,7 +975,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -966,7 +986,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -977,7 +997,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -988,7 +1008,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -1001,13 +1021,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1018,7 +1038,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1029,7 +1049,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1040,7 +1060,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1051,7 +1071,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1062,7 +1082,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1073,7 +1093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1093,13 +1113,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1110,7 +1130,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1121,7 +1141,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1132,7 +1152,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1143,7 +1163,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1154,7 +1174,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1165,7 +1185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1185,13 +1205,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1202,7 +1222,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1213,7 +1233,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1224,7 +1244,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1235,7 +1255,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1246,7 +1266,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1257,7 +1277,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1276,14 +1296,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1294,7 +1314,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>96</v>
       </c>
@@ -1305,7 +1325,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1316,7 +1336,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -1327,7 +1347,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1338,7 +1358,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1349,7 +1369,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -1360,7 +1380,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>96</v>
       </c>
@@ -1371,7 +1391,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>96</v>
       </c>
@@ -1382,7 +1402,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1393,7 +1413,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1404,7 +1424,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -1415,7 +1435,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -1426,7 +1446,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>96</v>
       </c>
@@ -1437,7 +1457,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1448,7 +1468,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -1459,7 +1479,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -1470,7 +1490,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -1481,7 +1501,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1492,7 +1512,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>96</v>
       </c>
@@ -1511,14 +1531,14 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.4609375" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1529,7 +1549,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1547,16 +1567,285 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA07446E-9ABB-4F29-9369-3956596EEF02}">
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>96</v>
+      </c>
+      <c r="B20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D129DC11-C1B5-4223-BFC6-17C380973951}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1567,7 +1856,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1578,7 +1867,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1589,7 +1878,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1600,7 +1889,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1617,16 +1906,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.4609375" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1637,7 +1926,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1648,7 +1937,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1659,7 +1948,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1672,126 +1961,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.07421875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.07421875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1802,7 +1984,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1813,7 +1995,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1824,7 +2006,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1835,7 +2017,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1846,10 +2028,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
     </row>
@@ -1860,16 +2042,16 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1880,180 +2062,37 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>96</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>96</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>96</v>
-      </c>
-      <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>96</v>
-      </c>
-      <c r="B11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>96</v>
-      </c>
-      <c r="B12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>96</v>
-      </c>
-      <c r="B13" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A15" t="s">
-        <v>96</v>
-      </c>
-      <c r="B15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A16" t="s">
-        <v>96</v>
-      </c>
-      <c r="B16" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A17" t="s">
-        <v>96</v>
-      </c>
-      <c r="B17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C17" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -2062,214 +2101,64 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
-  <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.4609375" customWidth="1"/>
-    <col min="2" max="2" width="9.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.3046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.07421875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.4609375" customWidth="1"/>
-    <col min="7" max="7" width="13.4609375" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3">
         <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.4">
-      <c r="E17" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.4">
-      <c r="E18" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.4">
-      <c r="E19" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
-      <c r="E20" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
-      <c r="E21" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.84375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2280,136 +2169,180 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>96</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>89</v>
-      </c>
-      <c r="C7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>93</v>
-      </c>
-      <c r="C11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C13" t="s">
-        <v>38</v>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2418,15 +2351,371 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E20" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2437,7 +2726,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2448,7 +2737,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2459,7 +2748,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2470,7 +2759,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2481,7 +2770,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2492,7 +2781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2509,17 +2798,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.84375" customWidth="1"/>
-    <col min="2" max="2" width="32.69140625" customWidth="1"/>
-    <col min="3" max="3" width="49.84375" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="32.6640625" customWidth="1"/>
+    <col min="3" max="3" width="49.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2530,7 +2819,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2541,7 +2830,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2552,7 +2841,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2563,7 +2852,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2574,7 +2863,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2585,7 +2874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2594,190 +2883,6 @@
       </c>
       <c r="C7">
         <v>3700</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="1" width="24.69140625" customWidth="1"/>
-    <col min="2" max="2" width="28.4609375" customWidth="1"/>
-    <col min="3" max="3" width="29.3046875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>365</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="1" width="27.84375" customWidth="1"/>
-    <col min="2" max="2" width="34.07421875" customWidth="1"/>
-    <col min="3" max="3" width="29.3046875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -2786,15 +2891,199 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28.44140625" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.88671875" customWidth="1"/>
+    <col min="2" max="2" width="34.109375" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2805,7 +3094,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2816,7 +3105,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2827,7 +3116,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2838,7 +3127,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2849,7 +3138,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2860,7 +3149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2877,197 +3166,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>365</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="2" max="2" width="11.84375" customWidth="1"/>
-    <col min="3" max="3" width="24.69140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>365</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.07421875" customWidth="1"/>
-    <col min="3" max="3" width="38.84375" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3078,7 +3186,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3089,7 +3197,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3100,7 +3208,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3111,7 +3219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3122,7 +3230,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3133,7 +3241,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3144,7 +3252,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3155,7 +3263,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3166,7 +3274,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -3178,15 +3286,14 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3197,7 +3304,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3208,7 +3315,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3216,10 +3323,10 @@
         <v>11</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3230,7 +3337,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3241,7 +3348,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3249,10 +3356,10 @@
         <v>102</v>
       </c>
       <c r="C6">
-        <v>-10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3269,15 +3376,15 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F3B454-4DBA-4E9B-A949-C34CD2C245D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3288,7 +3395,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3299,7 +3406,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3310,7 +3417,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3321,7 +3428,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3332,7 +3439,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3343,7 +3450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3351,7 +3458,7 @@
         <v>101</v>
       </c>
       <c r="C7">
-        <v>480</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -3360,15 +3467,15 @@
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268CDBE-0606-4B65-A8F6-04136D2C40DC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3379,7 +3486,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3390,18 +3497,200 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
+      <c r="C3" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F3B454-4DBA-4E9B-A949-C34CD2C245D5}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>480</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268CDBE-0606-4B65-A8F6-04136D2C40DC}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
       <c r="C3" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3412,7 +3701,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3423,7 +3712,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3434,7 +3723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3453,13 +3742,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3470,7 +3759,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3481,7 +3770,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3492,7 +3781,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3503,7 +3792,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3514,7 +3803,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3525,7 +3814,7 @@
         <v>-300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3544,14 +3833,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.69140625" customWidth="1"/>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3562,7 +3851,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3573,7 +3862,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3584,7 +3873,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3595,7 +3884,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3606,7 +3895,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3617,7 +3906,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3628,7 +3917,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3639,7 +3928,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3650,7 +3939,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3661,7 +3950,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3672,7 +3961,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3683,7 +3972,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3703,14 +3992,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2831158A-D169-49BB-9942-2243EC476E43}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.69140625" customWidth="1"/>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3721,7 +4010,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3732,7 +4021,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3743,7 +4032,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3754,7 +4043,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3765,7 +4054,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3776,7 +4065,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3787,7 +4076,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3798,7 +4087,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3809,7 +4098,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3820,7 +4109,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3831,7 +4120,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3842,7 +4131,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3861,13 +4150,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.53515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -3878,7 +4167,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3889,7 +4178,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3900,7 +4189,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -3911,7 +4200,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -3922,7 +4211,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -3933,7 +4222,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -3949,14 +4238,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3967,7 +4256,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3978,13 +4267,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C5" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
         <v>114</v>
       </c>
@@ -3998,14 +4287,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4016,7 +4305,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -4027,7 +4316,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>81</v>
       </c>

</xml_diff>

<commit_message>
Fixed failed testc ases
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Product Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D32CBE5-93AD-4D54-924F-0D62D0587695}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D15A67-E5D6-43EE-8A38-99F27B49DAB1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="8" activeTab="11" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="3" activeTab="9" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -22,29 +22,30 @@
     <sheet name="Sheet3" sheetId="14" r:id="rId7"/>
     <sheet name="Edition" sheetId="1" r:id="rId8"/>
     <sheet name="Edition_StandAlone" sheetId="9" r:id="rId9"/>
-    <sheet name="Grant_Creation1" sheetId="31" r:id="rId10"/>
-    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId11"/>
-    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId12"/>
-    <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId13"/>
-    <sheet name="Risk Assessment" sheetId="4" r:id="rId14"/>
-    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId15"/>
-    <sheet name="Reviewer" sheetId="6" r:id="rId16"/>
-    <sheet name="Site Visit" sheetId="5" r:id="rId17"/>
-    <sheet name="Desk Review" sheetId="7" r:id="rId18"/>
-    <sheet name="KPI" sheetId="18" r:id="rId19"/>
-    <sheet name="Risk Assessment1" sheetId="29" r:id="rId20"/>
-    <sheet name="Sheet1" sheetId="8" r:id="rId21"/>
-    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId22"/>
-    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId23"/>
-    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId24"/>
-    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId25"/>
-    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId26"/>
-    <sheet name="Progress Report Annually" sheetId="24" r:id="rId27"/>
-    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId28"/>
-    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId29"/>
-    <sheet name="Progress Report StartDate Error" sheetId="32" r:id="rId30"/>
-    <sheet name="Progress Report MoreThanOneyear" sheetId="33" r:id="rId31"/>
-    <sheet name="ProgressReportQuartelyReporting" sheetId="34" r:id="rId32"/>
+    <sheet name="Grant_Creation3" sheetId="35" r:id="rId10"/>
+    <sheet name="Grant_Creation1" sheetId="31" r:id="rId11"/>
+    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId12"/>
+    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId13"/>
+    <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId14"/>
+    <sheet name="Risk Assessment" sheetId="4" r:id="rId15"/>
+    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId16"/>
+    <sheet name="Reviewer" sheetId="6" r:id="rId17"/>
+    <sheet name="Site Visit" sheetId="5" r:id="rId18"/>
+    <sheet name="Desk Review" sheetId="7" r:id="rId19"/>
+    <sheet name="KPI" sheetId="18" r:id="rId20"/>
+    <sheet name="Risk Assessment1" sheetId="29" r:id="rId21"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId22"/>
+    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId23"/>
+    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId24"/>
+    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId25"/>
+    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId26"/>
+    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId27"/>
+    <sheet name="Progress Report Annually" sheetId="24" r:id="rId28"/>
+    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId29"/>
+    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId30"/>
+    <sheet name="Progress Report StartDate Error" sheetId="32" r:id="rId31"/>
+    <sheet name="Progress Report MoreThanOneyear" sheetId="33" r:id="rId32"/>
+    <sheet name="ProgressReportQuartelyReporting" sheetId="34" r:id="rId33"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -56,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="123">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -422,13 +423,16 @@
   </si>
   <si>
     <t>Automation Payment Request</t>
+  </si>
+  <si>
+    <t>Bayside Community Center</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -465,6 +469,13 @@
       <color rgb="FF333333"/>
       <name val="Helvetica"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF297BDE"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -486,7 +497,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -504,6 +515,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -819,13 +833,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -836,7 +850,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -847,7 +861,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -858,7 +872,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -869,7 +883,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -887,15 +901,134 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AA15B4A-9A74-424C-B76B-FE1349821083}">
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G19" t="s">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
-    <col min="3" max="3" width="38.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -906,7 +1039,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -917,7 +1050,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -928,7 +1061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -939,7 +1072,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -950,7 +1083,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -961,7 +1094,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -972,7 +1105,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -983,7 +1116,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -994,7 +1127,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G19" t="s">
         <v>116</v>
       </c>
@@ -1004,16 +1137,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1024,7 +1157,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1035,7 +1168,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1046,7 +1179,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1057,7 +1190,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1068,7 +1201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1079,7 +1212,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1096,16 +1229,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1116,7 +1249,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1127,7 +1260,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1138,7 +1271,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1149,7 +1282,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1160,7 +1293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1171,7 +1304,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1188,16 +1321,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1208,7 +1341,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1219,7 +1352,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1230,7 +1363,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1241,7 +1374,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1252,7 +1385,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1263,7 +1396,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1272,241 +1405,6 @@
       </c>
       <c r="C7">
         <v>3650</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
-  <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>96</v>
-      </c>
-      <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>96</v>
-      </c>
-      <c r="B11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>96</v>
-      </c>
-      <c r="B12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>96</v>
-      </c>
-      <c r="B13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>96</v>
-      </c>
-      <c r="B15" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>96</v>
-      </c>
-      <c r="B16" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>96</v>
-      </c>
-      <c r="B17" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>96</v>
-      </c>
-      <c r="B18" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>96</v>
-      </c>
-      <c r="B19" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>96</v>
-      </c>
-      <c r="B20" t="s">
-        <v>49</v>
-      </c>
-      <c r="C20" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1515,16 +1413,251 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>96</v>
+      </c>
+      <c r="B20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1535,7 +1668,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1552,17 +1685,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1573,7 +1706,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1584,7 +1717,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1595,7 +1728,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1606,7 +1739,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1623,16 +1756,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1643,7 +1776,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1654,7 +1787,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1665,66 +1798,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1741,15 +1815,16 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.140625" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1760,44 +1835,54 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
+      <c r="B3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1808,7 +1893,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1819,7 +1904,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1830,7 +1915,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1841,7 +1926,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1852,10 +1937,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="4"/>
     </row>
@@ -1866,16 +1951,15 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1886,379 +1970,229 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>96</v>
-      </c>
-      <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>96</v>
-      </c>
-      <c r="B11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>96</v>
-      </c>
-      <c r="B12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>96</v>
-      </c>
-      <c r="B13" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>96</v>
-      </c>
-      <c r="B15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>96</v>
-      </c>
-      <c r="B16" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>96</v>
-      </c>
-      <c r="B17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C17" t="s">
-        <v>48</v>
+        <v>9</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
-  <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>96</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>96</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E17" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E18" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E19" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E20" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E21" t="s">
-        <v>51</v>
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2267,155 +2201,197 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>89</v>
-      </c>
-      <c r="C7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>93</v>
-      </c>
-      <c r="C11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C13" t="s">
-        <v>38</v>
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E20" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E21" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -2424,15 +2400,172 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2443,7 +2576,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2454,7 +2587,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2465,7 +2598,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2476,7 +2609,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2487,7 +2620,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2498,7 +2631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2515,17 +2648,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="32.7109375" customWidth="1"/>
-    <col min="3" max="3" width="49.85546875" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="32.6640625" customWidth="1"/>
+    <col min="3" max="3" width="49.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2536,7 +2669,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2547,7 +2680,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2558,7 +2691,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2569,7 +2702,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2580,7 +2713,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2591,7 +2724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2600,98 +2733,6 @@
       </c>
       <c r="C7">
         <v>3700</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
-    <col min="2" max="2" width="28.42578125" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -2700,16 +2741,16 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.85546875" customWidth="1"/>
-    <col min="2" max="2" width="34.140625" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28.44140625" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2720,7 +2761,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2731,7 +2772,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2739,10 +2780,10 @@
         <v>11</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2753,7 +2794,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2764,7 +2805,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2775,7 +2816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2792,15 +2833,107 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.88671875" customWidth="1"/>
+    <col min="2" max="2" width="34.109375" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2811,7 +2944,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2822,7 +2955,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2833,7 +2966,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2844,7 +2977,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2855,7 +2988,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2866,7 +2999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2883,15 +3016,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2902,7 +3035,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2913,7 +3046,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2924,7 +3057,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2935,7 +3068,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2946,7 +3079,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2957,98 +3090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>365</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="11.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3067,13 +3109,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
-    <col min="3" max="3" width="38.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="3" max="3" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3084,7 +3126,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3095,7 +3137,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3106,7 +3148,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3117,7 +3159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3128,7 +3170,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3139,7 +3181,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3150,7 +3192,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3161,7 +3203,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3172,7 +3214,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G20" t="s">
         <v>116</v>
       </c>
@@ -3184,15 +3226,15 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3203,7 +3245,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3214,7 +3256,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3225,7 +3267,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3236,7 +3278,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3247,7 +3289,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3255,10 +3297,10 @@
         <v>102</v>
       </c>
       <c r="C6">
-        <v>-10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3275,15 +3317,15 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F3B454-4DBA-4E9B-A949-C34CD2C245D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3294,7 +3336,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3305,7 +3347,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3316,7 +3358,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3327,7 +3369,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3338,7 +3380,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3346,10 +3388,10 @@
         <v>102</v>
       </c>
       <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3357,7 +3399,7 @@
         <v>101</v>
       </c>
       <c r="C7">
-        <v>480</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -3366,15 +3408,15 @@
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268CDBE-0606-4B65-A8F6-04136D2C40DC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F3B454-4DBA-4E9B-A949-C34CD2C245D5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3385,7 +3427,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3396,18 +3438,109 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
+      <c r="C3" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>480</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268CDBE-0606-4B65-A8F6-04136D2C40DC}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
       <c r="C3" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3418,7 +3551,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3429,7 +3562,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3440,7 +3573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3459,13 +3592,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3476,7 +3609,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3487,7 +3620,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3498,7 +3631,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3509,7 +3642,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3520,7 +3653,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3531,7 +3664,7 @@
         <v>-300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3550,14 +3683,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3568,7 +3701,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3579,7 +3712,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3590,7 +3723,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3601,7 +3734,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3612,7 +3745,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3623,7 +3756,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3634,7 +3767,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3645,7 +3778,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3656,7 +3789,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3667,7 +3800,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3678,7 +3811,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3689,7 +3822,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3709,14 +3842,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2831158A-D169-49BB-9942-2243EC476E43}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3727,7 +3860,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3738,7 +3871,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3749,7 +3882,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3760,7 +3893,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3771,7 +3904,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3782,7 +3915,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -3793,7 +3926,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -3804,7 +3937,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -3815,7 +3948,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -3826,7 +3959,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -3837,7 +3970,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -3848,7 +3981,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -3867,13 +4000,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -3884,7 +4017,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3895,7 +4028,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3906,7 +4039,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
@@ -3917,7 +4050,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -3928,7 +4061,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -3939,7 +4072,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -3955,14 +4088,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3973,7 +4106,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -3984,13 +4117,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C5" s="6"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
         <v>114</v>
       </c>
@@ -4004,14 +4137,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4022,7 +4155,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -4033,7 +4166,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>81</v>
       </c>

</xml_diff>

<commit_message>
Added 4 TC and Run Failed Test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,52 +1,54 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Automation_Product\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615393D1-7DA7-4B7F-83CB-D6C59D65E45F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B47F408-299B-43C2-9135-3F6BF40AB467}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="3" activeTab="9" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="2" activeTab="3" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
     <sheet name="Payment Request Schedule_FDM" sheetId="15" r:id="rId2"/>
     <sheet name="Grant_Creation" sheetId="10" r:id="rId3"/>
-    <sheet name="Progress Report Error" sheetId="27" r:id="rId4"/>
-    <sheet name="Grant_Edition" sheetId="11" r:id="rId5"/>
-    <sheet name="Grant_Edition1" sheetId="30" r:id="rId6"/>
-    <sheet name="Sheet3" sheetId="14" r:id="rId7"/>
-    <sheet name="Edition" sheetId="1" r:id="rId8"/>
-    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId9"/>
-    <sheet name="Grant_Creation4" sheetId="36" r:id="rId10"/>
-    <sheet name="Grant_Creation3" sheetId="35" r:id="rId11"/>
-    <sheet name="Grant_Creation1" sheetId="31" r:id="rId12"/>
-    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId13"/>
-    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId14"/>
-    <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId15"/>
-    <sheet name="Risk Assessment" sheetId="4" r:id="rId16"/>
-    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId17"/>
-    <sheet name="Reviewer" sheetId="6" r:id="rId18"/>
-    <sheet name="Site Visit" sheetId="5" r:id="rId19"/>
-    <sheet name="Desk Review" sheetId="7" r:id="rId20"/>
-    <sheet name="KPI" sheetId="18" r:id="rId21"/>
-    <sheet name="Risk Assessment1" sheetId="29" r:id="rId22"/>
-    <sheet name="Sheet1" sheetId="8" r:id="rId23"/>
-    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId24"/>
-    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId25"/>
-    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId26"/>
-    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId27"/>
-    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId28"/>
-    <sheet name="Progress Report Annually" sheetId="24" r:id="rId29"/>
-    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId30"/>
-    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId31"/>
-    <sheet name="Progress Report StartDate Error" sheetId="32" r:id="rId32"/>
-    <sheet name="Progress Report MoreThanOneyear" sheetId="33" r:id="rId33"/>
-    <sheet name="ProgressReportQuartelyReporting" sheetId="34" r:id="rId34"/>
+    <sheet name="Grant_Creation_Error_2" sheetId="38" r:id="rId4"/>
+    <sheet name="Grant_Creation_Title_Error" sheetId="37" r:id="rId5"/>
+    <sheet name="Progress Report Error" sheetId="27" r:id="rId6"/>
+    <sheet name="Grant_Edition" sheetId="11" r:id="rId7"/>
+    <sheet name="Grant_Edition1" sheetId="30" r:id="rId8"/>
+    <sheet name="Sheet3" sheetId="14" r:id="rId9"/>
+    <sheet name="Edition" sheetId="1" r:id="rId10"/>
+    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId11"/>
+    <sheet name="Grant_Creation4" sheetId="36" r:id="rId12"/>
+    <sheet name="Grant_Creation3" sheetId="35" r:id="rId13"/>
+    <sheet name="Grant_Creation1" sheetId="31" r:id="rId14"/>
+    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId15"/>
+    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId16"/>
+    <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId17"/>
+    <sheet name="Risk Assessment" sheetId="4" r:id="rId18"/>
+    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId19"/>
+    <sheet name="Reviewer" sheetId="6" r:id="rId20"/>
+    <sheet name="Site Visit" sheetId="5" r:id="rId21"/>
+    <sheet name="Desk Review" sheetId="7" r:id="rId22"/>
+    <sheet name="KPI" sheetId="18" r:id="rId23"/>
+    <sheet name="Risk Assessment1" sheetId="29" r:id="rId24"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId25"/>
+    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId26"/>
+    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId27"/>
+    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId28"/>
+    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId29"/>
+    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId30"/>
+    <sheet name="Progress Report Annually" sheetId="24" r:id="rId31"/>
+    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId32"/>
+    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId33"/>
+    <sheet name="Progress Report StartDate Error" sheetId="32" r:id="rId34"/>
+    <sheet name="Progress Report MoreThanOneyear" sheetId="33" r:id="rId35"/>
+    <sheet name="ProgressReportQuartelyReporting" sheetId="34" r:id="rId36"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -58,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="125">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -867,10 +869,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -935,13 +937,110 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="16.6328125" customWidth="1"/>
+    <col min="2" max="2" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="C4" s="5"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="C5" s="6"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="D7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="16.6328125" customWidth="1"/>
+    <col min="2" max="2" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF806FA6-453F-48DB-A77C-F9ADAC509201}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1049,13 +1148,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AA15B4A-9A74-424C-B76B-FE1349821083}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
-    <col min="3" max="3" width="38.88671875" customWidth="1"/>
+    <col min="2" max="2" width="26.08984375" customWidth="1"/>
+    <col min="3" max="3" width="38.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1174,13 +1273,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
-    <col min="3" max="3" width="38.88671875" customWidth="1"/>
+    <col min="2" max="2" width="26.08984375" customWidth="1"/>
+    <col min="3" max="3" width="38.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1292,13 +1391,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1384,13 +1483,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1476,10 +1575,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -1567,14 +1666,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1802,14 +1901,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1840,142 +1939,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2047,13 +2017,13 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2072,10 +2042,80 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="2" max="2" width="21.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
         <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2105,13 +2145,72 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" customWidth="1"/>
+    <col min="2" max="2" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2153,14 +2252,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2348,362 +2447,6 @@
       </c>
       <c r="C17" t="s">
         <v>48</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
-  <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="E11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="E12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="E13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="E14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="E15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="E16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="5:5">
-      <c r="E17" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="5:5">
-      <c r="E18" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="5:5">
-      <c r="E19" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="5:5">
-      <c r="E20" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="5:5">
-      <c r="E21" t="s">
-        <v>51</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>89</v>
-      </c>
-      <c r="C7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>93</v>
-      </c>
-      <c r="C11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C13" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -2712,12 +2455,368 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="14.453125" customWidth="1"/>
+    <col min="2" max="2" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.453125" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="5:5">
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="5:5">
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="5:5">
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="5:5">
+      <c r="E20" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="5:5">
+      <c r="E21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2803,14 +2902,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" customWidth="1"/>
-    <col min="2" max="2" width="32.6640625" customWidth="1"/>
-    <col min="3" max="3" width="49.88671875" customWidth="1"/>
+    <col min="1" max="1" width="18.90625" customWidth="1"/>
+    <col min="2" max="2" width="32.6328125" customWidth="1"/>
+    <col min="3" max="3" width="49.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2888,190 +2987,6 @@
       </c>
       <c r="C7">
         <v>3700</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="24.6640625" customWidth="1"/>
-    <col min="2" max="2" width="28.44140625" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>365</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="27.88671875" customWidth="1"/>
-    <col min="2" max="2" width="34.109375" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -3080,9 +2995,312 @@
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="24.6328125" customWidth="1"/>
+    <col min="2" max="2" width="28.453125" customWidth="1"/>
+    <col min="3" max="3" width="29.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="2" max="2" width="26.08984375" customWidth="1"/>
+    <col min="3" max="3" width="38.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="7:7">
+      <c r="G20" t="s">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="27.90625" customWidth="1"/>
+    <col min="2" max="2" width="34.08984375" customWidth="1"/>
+    <col min="3" max="3" width="29.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -3171,129 +3389,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
-  <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
-    <col min="3" max="3" width="38.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5">
-        <v>3650</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C8" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>77</v>
-      </c>
-      <c r="C9" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="20" spans="7:7">
-      <c r="G20" t="s">
-        <v>116</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
   </cols>
@@ -3380,13 +3479,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="11.88671875" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" customWidth="1"/>
+    <col min="3" max="3" width="24.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3471,10 +3570,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -3562,10 +3661,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F3B454-4DBA-4E9B-A949-C34CD2C245D5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -3653,10 +3752,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268CDBE-0606-4B65-A8F6-04136D2C40DC}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -3745,9 +3844,213 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2B1888C-E65A-4810-8D83-FD31C65A906B}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="42.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E2B3190-9B72-4370-B928-04A0753C7A8E}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="2" max="2" width="29.1796875" customWidth="1"/>
+    <col min="3" max="3" width="54.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
@@ -3835,14 +4138,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6328125" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3994,14 +4297,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2831158A-D169-49BB-9942-2243EC476E43}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6328125" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4152,13 +4455,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4238,101 +4541,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="C4" s="5"/>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="C5" s="6"/>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="D7" t="s">
-        <v>114</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="16.6640625" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3">
-        <v>3650</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
5 more new scenario added
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47A3820E-090E-458C-A3E3-00BF31AF97B0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91AF73CA-8E2D-415C-991C-298BD8088695}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="3" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="5" activeTab="6" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -19,41 +19,42 @@
     <sheet name="Payment Request Schedule_FDM" sheetId="15" r:id="rId4"/>
     <sheet name="Payment_Request_Wt_Frequency" sheetId="42" r:id="rId5"/>
     <sheet name="Grant_Creation" sheetId="10" r:id="rId6"/>
-    <sheet name="GrantFields1" sheetId="40" r:id="rId7"/>
-    <sheet name="GrantFields3" sheetId="43" r:id="rId8"/>
-    <sheet name="GrantFields2" sheetId="41" r:id="rId9"/>
-    <sheet name="Grant_Create_less_date" sheetId="39" r:id="rId10"/>
-    <sheet name="Progress Report Error" sheetId="27" r:id="rId11"/>
-    <sheet name="Grant_Edition" sheetId="11" r:id="rId12"/>
-    <sheet name="Grant_Edition1" sheetId="30" r:id="rId13"/>
-    <sheet name="Sheet3" sheetId="14" r:id="rId14"/>
-    <sheet name="Edition" sheetId="1" r:id="rId15"/>
-    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId16"/>
-    <sheet name="Grant_Creation4" sheetId="36" r:id="rId17"/>
-    <sheet name="Grant_Creation3" sheetId="35" r:id="rId18"/>
-    <sheet name="Grant_Creation1" sheetId="31" r:id="rId19"/>
-    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId20"/>
-    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId21"/>
-    <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId22"/>
-    <sheet name="Risk Assessment" sheetId="4" r:id="rId23"/>
-    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId24"/>
-    <sheet name="Reviewer" sheetId="6" r:id="rId25"/>
-    <sheet name="Site Visit" sheetId="5" r:id="rId26"/>
-    <sheet name="Desk Review" sheetId="7" r:id="rId27"/>
-    <sheet name="KPI" sheetId="18" r:id="rId28"/>
-    <sheet name="Risk Assessment1" sheetId="29" r:id="rId29"/>
-    <sheet name="Sheet1" sheetId="8" r:id="rId30"/>
-    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId31"/>
-    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId32"/>
-    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId33"/>
-    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId34"/>
-    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId35"/>
-    <sheet name="Progress Report Annually" sheetId="24" r:id="rId36"/>
-    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId37"/>
-    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId38"/>
-    <sheet name="Progress Report StartDate Error" sheetId="32" r:id="rId39"/>
-    <sheet name="Progress Report MoreThanOneyear" sheetId="33" r:id="rId40"/>
-    <sheet name="ProgressReportQuartelyReporting" sheetId="34" r:id="rId41"/>
+    <sheet name="Grant_CreationDate" sheetId="44" r:id="rId7"/>
+    <sheet name="GrantFields1" sheetId="40" r:id="rId8"/>
+    <sheet name="GrantFields3" sheetId="43" r:id="rId9"/>
+    <sheet name="GrantFields2" sheetId="41" r:id="rId10"/>
+    <sheet name="Grant_Create_less_date" sheetId="39" r:id="rId11"/>
+    <sheet name="Progress Report Error" sheetId="27" r:id="rId12"/>
+    <sheet name="Grant_Edition" sheetId="11" r:id="rId13"/>
+    <sheet name="Grant_Edition1" sheetId="30" r:id="rId14"/>
+    <sheet name="Sheet3" sheetId="14" r:id="rId15"/>
+    <sheet name="Edition" sheetId="1" r:id="rId16"/>
+    <sheet name="Edition_StandAlone" sheetId="9" r:id="rId17"/>
+    <sheet name="Grant_Creation4" sheetId="36" r:id="rId18"/>
+    <sheet name="Grant_Creation3" sheetId="35" r:id="rId19"/>
+    <sheet name="Grant_Creation1" sheetId="31" r:id="rId20"/>
+    <sheet name="Payment Request Schedule" sheetId="2" r:id="rId21"/>
+    <sheet name="Progress Report Schedule" sheetId="3" r:id="rId22"/>
+    <sheet name="Progress Report Fixed Date" sheetId="28" r:id="rId23"/>
+    <sheet name="Risk Assessment" sheetId="4" r:id="rId24"/>
+    <sheet name="Risk Assessment Creation" sheetId="12" r:id="rId25"/>
+    <sheet name="Reviewer" sheetId="6" r:id="rId26"/>
+    <sheet name="Site Visit" sheetId="5" r:id="rId27"/>
+    <sheet name="Desk Review" sheetId="7" r:id="rId28"/>
+    <sheet name="KPI" sheetId="18" r:id="rId29"/>
+    <sheet name="Risk Assessment1" sheetId="29" r:id="rId30"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId31"/>
+    <sheet name="AdvPaymentGrandEdition" sheetId="19" r:id="rId32"/>
+    <sheet name="ProgressReport_Edition" sheetId="20" r:id="rId33"/>
+    <sheet name="ScheduledEndDateAfterStartDate" sheetId="22" r:id="rId34"/>
+    <sheet name="Progress Report Quarterly" sheetId="21" r:id="rId35"/>
+    <sheet name="Progress Report BiMonthly" sheetId="23" r:id="rId36"/>
+    <sheet name="Progress Report Annually" sheetId="24" r:id="rId37"/>
+    <sheet name="Progress Report Semi-Annually" sheetId="25" r:id="rId38"/>
+    <sheet name="Progress Report Monthly" sheetId="26" r:id="rId39"/>
+    <sheet name="Progress Report StartDate Error" sheetId="32" r:id="rId40"/>
+    <sheet name="Progress Report MoreThanOneyear" sheetId="33" r:id="rId41"/>
+    <sheet name="ProgressReportQuartelyReporting" sheetId="34" r:id="rId42"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -65,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="961" uniqueCount="127">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -958,6 +959,120 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB6C3290-90D3-4091-A830-4534FC405EA9}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{044B56D1-696B-4348-B6D7-1D9D0FC3A624}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1066,7 +1181,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1157,7 +1272,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1316,7 +1431,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2831158A-D169-49BB-9942-2243EC476E43}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1474,7 +1589,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA1DF80-10FA-482E-96C0-ACB00E266B8C}">
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1562,7 +1677,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1611,7 +1726,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1659,7 +1774,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF806FA6-453F-48DB-A77C-F9ADAC509201}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1774,7 +1889,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AA15B4A-9A74-424C-B76B-FE1349821083}">
   <dimension ref="A1:G19"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1896,124 +2011,6 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
-  <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
-    <col min="3" max="3" width="38.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4">
-        <v>3650</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G19" t="s">
-        <v>116</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2175,6 +2172,124 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="3" width="38.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G19" t="s">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2266,7 +2381,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2358,7 +2473,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2449,7 +2564,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2684,7 +2799,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2722,7 +2837,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2793,7 +2908,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2851,7 +2966,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2910,7 +3025,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2955,208 +3070,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>96</v>
-      </c>
-      <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>96</v>
-      </c>
-      <c r="B11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>96</v>
-      </c>
-      <c r="B12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>96</v>
-      </c>
-      <c r="B13" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>96</v>
-      </c>
-      <c r="B15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>96</v>
-      </c>
-      <c r="B16" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>96</v>
-      </c>
-      <c r="B17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C17" t="s">
-        <v>48</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -3285,6 +3198,208 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="61.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3483,7 +3598,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3640,7 +3755,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3732,7 +3847,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3824,7 +3939,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3916,7 +4031,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4008,7 +4123,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4100,7 +4215,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4190,7 +4305,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4263,97 +4378,6 @@
       </c>
       <c r="C6">
         <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7">
-        <v>365</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6">
-        <v>-10</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4452,6 +4476,97 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F3B454-4DBA-4E9B-A949-C34CD2C245D5}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4542,7 +4657,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268CDBE-0606-4B65-A8F6-04136D2C40DC}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4695,7 +4810,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="26.140625" customWidth="1"/>
@@ -4801,11 +4916,6 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G20" t="s">
-        <v>116</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4813,6 +4923,119 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{668B3B47-A008-4655-9D40-94DF3D883784}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="25.42578125" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACE6FFDD-86CC-47A1-A159-E67815015993}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4925,7 +5148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D025DC8-BAFD-CD42-9FF2-51AA4DCC7B3B}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5037,118 +5260,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB6C3290-90D3-4091-A830-4534FC405EA9}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5">
-        <v>3650</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C8" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>77</v>
-      </c>
-      <c r="C9" t="s">
-        <v>78</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fixed 2 test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1707487-D40A-4AFF-9398-FF86AFB77609}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FACFB1A8-2F10-40EC-922C-6778B7CADCFA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="4" activeTab="5" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
@@ -457,7 +457,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -508,6 +508,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -529,7 +535,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -562,6 +568,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4978,7 +4987,7 @@
       <c r="B2" t="s">
         <v>69</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="16" t="s">
         <v>119</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed test cases: attachment
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22624"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jitendrapisal/rei/govgrants-product-automation/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C633B960-8FFF-404F-B171-E803490B9E47}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8860FAD5-1400-2A4D-8586-60D9C04D35AC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="22140" windowHeight="11940" xr2:uid="{10FEA7AB-10C6-4A3F-BF77-BE44F0EFE02D}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1019" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="124">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -445,7 +445,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -873,14 +873,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62ACE97-36F7-4E73-A259-A264DD733BB1}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="21.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -891,7 +891,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -902,7 +902,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -913,7 +913,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -922,17 +922,6 @@
       </c>
       <c r="C4" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -944,14 +933,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB6C3290-90D3-4091-A830-4534FC405EA9}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.84375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -962,7 +951,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -973,7 +962,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -984,7 +973,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -995,7 +984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1006,7 +995,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1017,7 +1006,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1028,7 +1017,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1039,7 +1028,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1058,13 +1047,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{044B56D1-696B-4348-B6D7-1D9D0FC3A624}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.84375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1075,7 +1064,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1086,7 +1075,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1097,7 +1086,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1108,7 +1097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1119,7 +1108,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1130,7 +1119,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1141,7 +1130,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1152,7 +1141,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1171,13 +1160,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A057E164-C642-4069-AA67-BFDDC1682771}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1188,7 +1177,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1199,7 +1188,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1210,7 +1199,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1221,7 +1210,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1232,7 +1221,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1243,7 +1232,7 @@
         <v>-300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1262,14 +1251,14 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69DD06D-7A8F-4C83-860C-E6A58CC62982}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.69140625" customWidth="1"/>
-    <col min="2" max="2" width="29.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1280,7 +1269,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1291,7 +1280,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1302,7 +1291,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1313,7 +1302,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1324,7 +1313,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1335,7 +1324,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1346,7 +1335,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1357,7 +1346,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1368,7 +1357,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1379,7 +1368,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1390,7 +1379,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1401,7 +1390,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1421,14 +1410,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{898314A1-D73D-489D-81D2-2377E363BA20}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1439,7 +1428,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1450,7 +1439,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1461,7 +1450,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1472,7 +1461,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1483,7 +1472,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1494,7 +1483,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1505,7 +1494,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1516,7 +1505,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1527,7 +1516,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1538,7 +1527,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1549,7 +1538,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1560,7 +1549,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1571,7 +1560,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -1590,13 +1579,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{349898A8-8098-4551-AF70-D3DA338543E8}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.84375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1607,7 +1596,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1618,7 +1607,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1629,7 +1618,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1640,7 +1629,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1651,7 +1640,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1662,7 +1651,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1673,7 +1662,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1684,7 +1673,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1695,7 +1684,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1706,7 +1695,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1717,7 +1706,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1728,7 +1717,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1747,14 +1736,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2831158A-D169-49BB-9942-2243EC476E43}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.69140625" customWidth="1"/>
-    <col min="2" max="2" width="29.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1765,7 +1754,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1776,7 +1765,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1787,7 +1776,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1798,7 +1787,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1809,7 +1798,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1820,7 +1809,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1831,7 +1820,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1842,7 +1831,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1853,7 +1842,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1864,7 +1853,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1875,7 +1864,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1886,7 +1875,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1905,14 +1894,14 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27973165-7DE8-4261-971F-5AF0868835AC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1923,7 +1912,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1934,13 +1923,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4">
       <c r="C4" s="4"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4">
       <c r="C5" s="5"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4">
       <c r="D7" t="s">
         <v>105</v>
       </c>
@@ -1954,14 +1943,14 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D74D1B-C955-4ECC-9715-1FCC698B0F13}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.69140625" customWidth="1"/>
-    <col min="2" max="2" width="23.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1972,7 +1961,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1983,7 +1972,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>77</v>
       </c>
@@ -2002,14 +1991,14 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF806FA6-453F-48DB-A77C-F9ADAC509201}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2020,7 +2009,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2031,7 +2020,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2042,7 +2031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2053,7 +2042,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2064,7 +2053,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2075,7 +2064,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2086,7 +2075,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2097,7 +2086,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -2117,13 +2106,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2004B323-1D53-4498-A3AF-7A7A004D18A4}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2134,7 +2123,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2145,7 +2134,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2156,7 +2145,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2167,7 +2156,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2178,7 +2167,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2189,7 +2178,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2200,7 +2189,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2211,7 +2200,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -2222,7 +2211,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -2233,7 +2222,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -2244,7 +2233,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -2255,7 +2244,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -2274,13 +2263,13 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AA15B4A-9A74-424C-B76B-FE1349821083}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.07421875" customWidth="1"/>
-    <col min="3" max="3" width="38.84375" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2291,7 +2280,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2302,7 +2291,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2313,7 +2302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2324,7 +2313,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2335,7 +2324,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2346,7 +2335,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2357,7 +2346,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2368,7 +2357,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -2379,10 +2368,10 @@
         <v>117</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3">
       <c r="C10" s="8"/>
     </row>
-    <row r="19" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="19" spans="7:7">
       <c r="G19" t="s">
         <v>107</v>
       </c>
@@ -2399,13 +2388,13 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF9EC96-B84F-4905-9DD7-95EF3BF23A01}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.07421875" customWidth="1"/>
-    <col min="3" max="3" width="38.84375" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2416,7 +2405,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2427,7 +2416,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2438,7 +2427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2449,7 +2438,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2460,7 +2449,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2471,7 +2460,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2482,7 +2471,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -2493,7 +2482,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -2504,7 +2493,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="19" spans="7:7" x14ac:dyDescent="0.4">
+    <row r="19" spans="7:7">
       <c r="G19" t="s">
         <v>107</v>
       </c>
@@ -2517,13 +2506,13 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A9BCD66-1D37-42BA-8077-A6306C929076}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2534,7 +2523,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2545,7 +2534,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2556,7 +2545,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2567,7 +2556,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2578,7 +2567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2589,7 +2578,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2609,13 +2598,13 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99414344-EAF9-427C-9BB0-C0063BEEA389}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="21.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2626,7 +2615,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2637,7 +2626,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2648,7 +2637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2659,7 +2648,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2670,7 +2659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2681,7 +2670,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2701,13 +2690,13 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FAE8E0-2777-4BC9-8D4C-85DD911170A5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2718,7 +2707,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2729,7 +2718,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2740,7 +2729,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2751,7 +2740,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2762,7 +2751,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2773,7 +2762,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2792,14 +2781,14 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C0F4E67-C3F8-4D56-99A2-4C13A82795BC}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2810,7 +2799,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>89</v>
       </c>
@@ -2821,7 +2810,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>89</v>
       </c>
@@ -2832,7 +2821,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>89</v>
       </c>
@@ -2843,7 +2832,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>89</v>
       </c>
@@ -2854,7 +2843,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>89</v>
       </c>
@@ -2865,7 +2854,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>89</v>
       </c>
@@ -2876,7 +2865,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>89</v>
       </c>
@@ -2887,7 +2876,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>89</v>
       </c>
@@ -2898,7 +2887,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>89</v>
       </c>
@@ -2909,7 +2898,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>89</v>
       </c>
@@ -2920,7 +2909,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>89</v>
       </c>
@@ -2931,7 +2920,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>89</v>
       </c>
@@ -2942,7 +2931,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -2953,7 +2942,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>89</v>
       </c>
@@ -2964,7 +2953,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>89</v>
       </c>
@@ -2975,7 +2964,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>89</v>
       </c>
@@ -2986,7 +2975,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>89</v>
       </c>
@@ -2997,7 +2986,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>89</v>
       </c>
@@ -3008,7 +2997,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>89</v>
       </c>
@@ -3027,14 +3016,14 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA439DA5-D0A5-4AAC-AAE2-4792499148E8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.3046875" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3045,7 +3034,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -3065,14 +3054,14 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C85660-11FF-42F8-8499-AE3BC3F291AB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3083,7 +3072,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -3094,7 +3083,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -3105,7 +3094,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -3116,7 +3105,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -3136,13 +3125,13 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4E8202-CEB6-47CB-B42D-44799C100468}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="21.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.3046875" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3153,7 +3142,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -3164,7 +3153,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -3175,7 +3164,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -3194,14 +3183,14 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9B08E7-9F9B-487C-8014-9A20D47C3661}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.3046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3212,7 +3201,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -3223,7 +3212,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -3234,7 +3223,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -3253,13 +3242,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB22FE06-6BB5-4AD3-99B5-1EB5C931464E}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="29.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3270,7 +3259,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -3281,7 +3270,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -3292,7 +3281,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -3303,7 +3292,7 @@
         <v>-3650</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -3314,7 +3303,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -3325,7 +3314,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -3336,7 +3325,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -3347,7 +3336,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -3358,7 +3347,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -3377,13 +3366,13 @@
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A47C31-D254-4F2E-A2A3-03DE0C58DF3D}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="14.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.07421875" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3394,7 +3383,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -3405,7 +3394,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -3425,14 +3414,14 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982A2D4F-725B-462F-A6F0-CD37025EE141}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="61.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3443,7 +3432,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>89</v>
       </c>
@@ -3454,7 +3443,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>89</v>
       </c>
@@ -3465,7 +3454,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>89</v>
       </c>
@@ -3476,7 +3465,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>89</v>
       </c>
@@ -3487,7 +3476,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>89</v>
       </c>
@@ -3498,7 +3487,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>89</v>
       </c>
@@ -3509,7 +3498,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>89</v>
       </c>
@@ -3520,7 +3509,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>89</v>
       </c>
@@ -3531,7 +3520,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>89</v>
       </c>
@@ -3542,7 +3531,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>89</v>
       </c>
@@ -3553,7 +3542,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>89</v>
       </c>
@@ -3564,7 +3553,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>89</v>
       </c>
@@ -3575,7 +3564,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -3586,7 +3575,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>89</v>
       </c>
@@ -3597,7 +3586,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>89</v>
       </c>
@@ -3608,7 +3597,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>89</v>
       </c>
@@ -3627,18 +3616,18 @@
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B322793F-1508-4954-A96D-E508DE6F98E2}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.3046875" customWidth="1"/>
-    <col min="2" max="2" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="10.3046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.07421875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.3046875" customWidth="1"/>
-    <col min="7" max="7" width="13.3046875" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -3661,7 +3650,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3684,7 +3673,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -3704,7 +3693,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -3724,7 +3713,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3738,82 +3727,82 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7">
       <c r="E6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7">
       <c r="E7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7">
       <c r="E8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7">
       <c r="E9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7">
       <c r="E10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7">
       <c r="E11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7">
       <c r="E12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7">
       <c r="E13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7">
       <c r="E14" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7">
       <c r="E15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7">
       <c r="E16" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="17" spans="5:5">
       <c r="E17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="18" spans="5:5">
       <c r="E18" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="5:5">
       <c r="E19" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="5:5">
       <c r="E20" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="5:5">
       <c r="E21" t="s">
         <v>50</v>
       </c>
@@ -3826,13 +3815,13 @@
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC78B46-40A0-4CB8-9763-6E7E631A0C48}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.84375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3843,7 +3832,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -3854,7 +3843,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -3865,7 +3854,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -3876,7 +3865,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -3887,7 +3876,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -3898,7 +3887,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -3909,7 +3898,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -3920,7 +3909,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -3931,7 +3920,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -3942,7 +3931,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -3953,7 +3942,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -3964,7 +3953,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -3983,13 +3972,13 @@
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41D0EB0-7F8B-4D12-B4E4-19E9A0280072}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="21.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.69140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4000,7 +3989,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4011,7 +4000,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4022,7 +4011,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4033,7 +4022,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4044,7 +4033,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4055,7 +4044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4075,14 +4064,14 @@
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0C57387-E763-4AE4-BC73-76B2CFD5660F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.84375" customWidth="1"/>
-    <col min="2" max="2" width="32.69140625" customWidth="1"/>
-    <col min="3" max="3" width="49.84375" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.6640625" customWidth="1"/>
+    <col min="3" max="3" width="49.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4093,7 +4082,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4104,7 +4093,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4115,7 +4104,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4126,7 +4115,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4137,7 +4126,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4148,7 +4137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4167,14 +4156,14 @@
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79D4D7BD-E259-420F-B57C-97553341CA40}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.69140625" customWidth="1"/>
-    <col min="2" max="2" width="28.3046875" customWidth="1"/>
-    <col min="3" max="3" width="29.3046875" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4185,7 +4174,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4196,7 +4185,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4207,7 +4196,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4218,7 +4207,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4229,7 +4218,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4240,7 +4229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4259,14 +4248,14 @@
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55B1D96-CAB9-429D-B308-AD4E2102C9F9}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.84375" customWidth="1"/>
-    <col min="2" max="2" width="34.07421875" customWidth="1"/>
-    <col min="3" max="3" width="29.3046875" customWidth="1"/>
+    <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4277,7 +4266,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4288,7 +4277,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4299,7 +4288,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4310,7 +4299,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4321,7 +4310,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4332,7 +4321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4351,13 +4340,13 @@
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7667ECB5-3242-40AD-A99C-E440169044C4}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4368,7 +4357,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4379,7 +4368,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4390,7 +4379,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4401,7 +4390,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4412,7 +4401,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4423,7 +4412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4443,13 +4432,13 @@
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F77D14-FAE8-4C97-9497-A25BE1D39BA7}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4460,7 +4449,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4471,7 +4460,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4482,7 +4471,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4493,7 +4482,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4504,7 +4493,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4515,7 +4504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4533,16 +4522,16 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB64170-7C6A-43D2-B9DF-131AC457E710}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.69140625" style="12"/>
-    <col min="2" max="2" width="19.3046875" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.07421875" style="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.69140625" style="12"/>
+    <col min="1" max="1" width="8.6640625" style="12"/>
+    <col min="2" max="2" width="19.33203125" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.6640625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4553,7 +4542,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" s="12" t="s">
         <v>8</v>
       </c>
@@ -4564,7 +4553,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" s="12" t="s">
         <v>8</v>
       </c>
@@ -4575,7 +4564,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" s="12" t="s">
         <v>8</v>
       </c>
@@ -4586,23 +4575,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="14"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="B7" s="14"/>
-      <c r="C7" s="15"/>
+    <row r="5" spans="1:3">
+      <c r="B5" s="14"/>
+      <c r="C5" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4613,13 +4588,13 @@
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7169A81-756B-4781-84B9-B53F8E72B1D8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="11.84375" customWidth="1"/>
-    <col min="3" max="3" width="24.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4630,7 +4605,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4641,7 +4616,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4652,7 +4627,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4663,7 +4638,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4674,7 +4649,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4685,7 +4660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4704,13 +4679,13 @@
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4DB144-605B-4F5E-B562-9E0F0423D523}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4721,7 +4696,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4732,7 +4707,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4743,7 +4718,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4754,7 +4729,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4765,7 +4740,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4776,7 +4751,7 @@
         <v>-25</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4795,13 +4770,13 @@
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F3B454-4DBA-4E9B-A949-C34CD2C245D5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4812,7 +4787,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4823,7 +4798,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4834,7 +4809,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4845,7 +4820,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4856,7 +4831,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4867,7 +4842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4886,13 +4861,13 @@
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268CDBE-0606-4B65-A8F6-04136D2C40DC}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4903,7 +4878,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4914,7 +4889,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4925,7 +4900,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4936,7 +4911,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4947,7 +4922,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4958,7 +4933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4977,15 +4952,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27C04786-5DC5-40FD-8EF4-0A4E5EC57EDB}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.3046875" style="12" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" style="12" customWidth="1"/>
     <col min="2" max="2" width="19" style="12" customWidth="1"/>
-    <col min="3" max="3" width="31.84375" style="12" customWidth="1"/>
-    <col min="4" max="16384" width="8.84375" style="12"/>
+    <col min="3" max="3" width="31.83203125" style="12" customWidth="1"/>
+    <col min="4" max="16384" width="8.83203125" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4996,7 +4971,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" s="12" t="s">
         <v>8</v>
       </c>
@@ -5007,7 +4982,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" s="12" t="s">
         <v>8</v>
       </c>
@@ -5018,7 +4993,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" s="12" t="s">
         <v>8</v>
       </c>
@@ -5037,13 +5012,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB900D6-DDA0-4FE5-BFF4-CF0C76900E85}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.07421875" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="46" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5054,7 +5029,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="16">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -5065,7 +5040,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -5076,7 +5051,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -5087,7 +5062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -5098,7 +5073,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -5109,7 +5084,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -5120,7 +5095,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -5131,7 +5106,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -5151,13 +5126,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{668B3B47-A008-4655-9D40-94DF3D883784}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="25.4609375" customWidth="1"/>
+    <col min="2" max="2" width="25.5" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5168,7 +5143,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -5179,7 +5154,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -5190,7 +5165,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -5201,7 +5176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -5212,7 +5187,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -5223,7 +5198,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -5234,7 +5209,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -5245,7 +5220,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -5264,13 +5239,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACE6FFDD-86CC-47A1-A159-E67815015993}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="29.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5281,7 +5256,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -5292,7 +5267,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -5303,7 +5278,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -5314,7 +5289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -5325,7 +5300,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -5336,7 +5311,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -5347,7 +5322,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -5358,7 +5333,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -5377,14 +5352,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D025DC8-BAFD-CD42-9FF2-51AA4DCC7B3B}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.4609375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.84375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -5395,7 +5370,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" s="11" t="s">
         <v>8</v>
       </c>
@@ -5406,7 +5381,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" s="11" t="s">
         <v>8</v>
       </c>
@@ -5417,7 +5392,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" s="11" t="s">
         <v>8</v>
       </c>
@@ -5428,7 +5403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" s="11" t="s">
         <v>8</v>
       </c>
@@ -5439,7 +5414,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" s="11" t="s">
         <v>8</v>
       </c>
@@ -5450,7 +5425,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" s="11" t="s">
         <v>8</v>
       </c>
@@ -5461,7 +5436,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" s="11" t="s">
         <v>8</v>
       </c>
@@ -5472,7 +5447,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" s="11" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
made changes in Grantor Business sanity feature file
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="465" windowWidth="20730" windowHeight="11760" activeTab="11"/>
+    <workbookView xWindow="0" yWindow="465" windowWidth="20730" windowHeight="11760" firstSheet="5" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="125">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -433,6 +433,9 @@
   </si>
   <si>
     <t xml:space="preserve">Automation Runtime Payment Request </t>
+  </si>
+  <si>
+    <t>fieldProjectTitle__c</t>
   </si>
 </sst>
 </file>
@@ -2470,7 +2473,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
       <c r="C9" t="s">
         <v>117</v>
@@ -4984,7 +4987,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
       <c r="C2" s="16" t="s">
         <v>116</v>

</xml_diff>

<commit_message>
Modified Risk Assesment and Payment request module
</commit_message>
<xml_diff>
--- a/src/main/resources/Award_Field_Values.xlsx
+++ b/src/main/resources/Award_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E41BE16E-469D-42F0-9A62-C9D8FD226CBD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5702FC4B-0332-4BF5-AAF0-425D4451B709}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="20" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="19" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Report Schedule_FDM" sheetId="16" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="128">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -236,9 +236,6 @@
     <t>Lookup</t>
   </si>
   <si>
-    <t>Automation SPI</t>
-  </si>
-  <si>
     <t>MonitoringType__c</t>
   </si>
   <si>
@@ -398,18 +395,12 @@
     <t>02/02/2024</t>
   </si>
   <si>
-    <t>Bayside Community Center</t>
-  </si>
-  <si>
     <t>InternalOrganization__c</t>
   </si>
   <si>
     <t>SYSTEM</t>
   </si>
   <si>
-    <t>St. Vincent De Paul Village, Inc.</t>
-  </si>
-  <si>
     <t>BudgetRedirectionThreshhold__c</t>
   </si>
   <si>
@@ -459,6 +450,9 @@
   </si>
   <si>
     <t>fieldExternalOrganization__c</t>
+  </si>
+  <si>
+    <t>Automation SPI3</t>
   </si>
 </sst>
 </file>
@@ -926,7 +920,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -937,7 +931,7 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -983,10 +977,10 @@
         <v>8</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -994,10 +988,10 @@
         <v>8</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -1005,7 +999,7 @@
         <v>8</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C4" s="11">
         <v>0</v>
@@ -1016,7 +1010,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C5" s="11">
         <v>3650</v>
@@ -1027,10 +1021,10 @@
         <v>8</v>
       </c>
       <c r="B6" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="11" t="s">
         <v>70</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -1038,10 +1032,10 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -1049,10 +1043,10 @@
         <v>8</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
@@ -1060,10 +1054,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1097,10 +1091,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -1108,10 +1102,10 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -1119,7 +1113,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1130,7 +1124,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -1141,10 +1135,10 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" t="s">
         <v>70</v>
-      </c>
-      <c r="C6" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -1152,10 +1146,10 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -1163,10 +1157,10 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
@@ -1174,10 +1168,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" t="s">
         <v>74</v>
-      </c>
-      <c r="C9" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1210,10 +1204,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -1221,10 +1215,10 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -1232,7 +1226,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1243,7 +1237,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C5">
         <v>365</v>
@@ -1254,10 +1248,10 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" t="s">
         <v>70</v>
-      </c>
-      <c r="C6" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -1265,10 +1259,10 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -1276,10 +1270,10 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
@@ -1287,10 +1281,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" t="s">
         <v>74</v>
-      </c>
-      <c r="C9" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1326,7 +1320,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -1337,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -1356,7 +1350,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C5">
         <v>-300</v>
@@ -1367,7 +1361,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C6">
         <v>1000</v>
@@ -1404,7 +1398,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C2" t="s">
         <v>37</v>
@@ -1415,7 +1409,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1426,7 +1420,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C4" t="s">
         <v>37</v>
@@ -1437,7 +1431,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
         <v>37</v>
@@ -1448,7 +1442,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
@@ -1459,7 +1453,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
         <v>30</v>
@@ -1470,7 +1464,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -1481,7 +1475,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
         <v>37</v>
@@ -1492,7 +1486,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" t="s">
         <v>37</v>
@@ -1503,7 +1497,7 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>37</v>
@@ -1514,7 +1508,7 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
         <v>30</v>
@@ -1525,7 +1519,7 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
         <v>37</v>
@@ -1563,7 +1557,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C2" t="s">
         <v>37</v>
@@ -1574,7 +1568,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1585,7 +1579,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C4" t="s">
         <v>37</v>
@@ -1596,7 +1590,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
         <v>37</v>
@@ -1607,7 +1601,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
@@ -1618,7 +1612,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
         <v>30</v>
@@ -1629,7 +1623,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -1640,7 +1634,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
         <v>37</v>
@@ -1651,7 +1645,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" t="s">
         <v>37</v>
@@ -1662,7 +1656,7 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>37</v>
@@ -1673,7 +1667,7 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
         <v>30</v>
@@ -1684,7 +1678,7 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
         <v>37</v>
@@ -1695,7 +1689,7 @@
         <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C14">
         <v>15</v>
@@ -1731,7 +1725,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C2" t="s">
         <v>37</v>
@@ -1742,7 +1736,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1753,7 +1747,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C4" t="s">
         <v>37</v>
@@ -1764,7 +1758,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
         <v>37</v>
@@ -1775,7 +1769,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
@@ -1786,7 +1780,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
         <v>30</v>
@@ -1797,7 +1791,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -1808,7 +1802,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
         <v>37</v>
@@ -1819,7 +1813,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" t="s">
         <v>30</v>
@@ -1830,7 +1824,7 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>37</v>
@@ -1841,7 +1835,7 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
         <v>30</v>
@@ -1852,7 +1846,7 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
         <v>37</v>
@@ -1889,7 +1883,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C2" t="s">
         <v>37</v>
@@ -1900,7 +1894,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1911,7 +1905,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C4" t="s">
         <v>37</v>
@@ -1922,7 +1916,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
         <v>37</v>
@@ -1933,7 +1927,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
@@ -1944,7 +1938,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
         <v>30</v>
@@ -1955,7 +1949,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -1966,7 +1960,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
         <v>37</v>
@@ -1977,7 +1971,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" t="s">
         <v>37</v>
@@ -1988,7 +1982,7 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>30</v>
@@ -1999,7 +1993,7 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
         <v>30</v>
@@ -2010,7 +2004,7 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
         <v>37</v>
@@ -2061,7 +2055,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="D7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2104,10 +2098,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C3">
         <v>3650</v>
@@ -2143,7 +2137,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C2" t="s">
         <v>37</v>
@@ -2154,7 +2148,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -2165,7 +2159,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C4" t="s">
         <v>37</v>
@@ -2176,7 +2170,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
         <v>37</v>
@@ -2187,7 +2181,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
@@ -2198,7 +2192,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
         <v>37</v>
@@ -2209,7 +2203,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -2220,7 +2214,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
         <v>37</v>
@@ -2231,7 +2225,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" t="s">
         <v>37</v>
@@ -2242,7 +2236,7 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>37</v>
@@ -2253,7 +2247,7 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
         <v>30</v>
@@ -2264,7 +2258,7 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
         <v>37</v>
@@ -2301,10 +2295,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -2312,7 +2306,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -2323,7 +2317,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C4">
         <v>3650</v>
@@ -2334,10 +2328,10 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" t="s">
         <v>70</v>
-      </c>
-      <c r="C5" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
@@ -2345,10 +2339,10 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
+      </c>
+      <c r="C6" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -2356,10 +2350,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -2367,10 +2361,10 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" t="s">
         <v>74</v>
-      </c>
-      <c r="C8" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
@@ -2378,10 +2372,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -2415,10 +2409,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -2426,7 +2420,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -2437,7 +2431,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C4">
         <v>3650</v>
@@ -2448,10 +2442,10 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" t="s">
         <v>70</v>
-      </c>
-      <c r="C5" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
@@ -2459,10 +2453,10 @@
         <v>8</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C6" t="s">
-        <v>112</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -2470,10 +2464,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -2481,10 +2475,10 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" t="s">
         <v>74</v>
-      </c>
-      <c r="C8" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
@@ -2492,10 +2486,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
@@ -2503,15 +2497,12 @@
     </row>
     <row r="19" spans="7:7" x14ac:dyDescent="0.45">
       <c r="G19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C6" r:id="rId1" tooltip="St. Vincent De Paul Village, Inc." display="https://test8-internal--automation--c.visualforce.com/0011800000qpsx9AAA" xr:uid="{00000000-0004-0000-1300-000000000000}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2540,10 +2531,10 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -2551,7 +2542,7 @@
         <v>8</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -2562,7 +2553,7 @@
         <v>8</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C4">
         <v>3650</v>
@@ -2573,10 +2564,10 @@
         <v>8</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C5" t="s"